<commit_message>
Design Platinum Block Parser Prompt 08 and update work diary
</commit_message>
<xml_diff>
--- a/OCR-NER-Pipeline-v3/output/generated-database-v4.xlsx
+++ b/OCR-NER-Pipeline-v3/output/generated-database-v4.xlsx
@@ -1261,7 +1261,11 @@
           <t>26/05/1970</t>
         </is>
       </c>
-      <c r="B2" s="30" t="inlineStr"/>
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>AO</t>
+        </is>
+      </c>
       <c r="C2" s="30" t="inlineStr">
         <is>
           <t>9990001</t>
@@ -1284,28 +1288,20 @@
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr"/>
-      <c r="I2" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J2" s="30" t="inlineStr">
-        <is>
-          <t>At 13cm from insertion there was a malignant looking mass with an abnormal pit pattern suspicious features for malignancy.</t>
-        </is>
-      </c>
+      <c r="I2" s="30" t="inlineStr"/>
+      <c r="J2" s="30" t="inlineStr"/>
       <c r="K2" s="30" t="inlineStr">
         <is>
           <t>ADENOCARCINOMA, NOT OTHERWISE SPECIFIED  ICD10 Code: 10 - C20: Malignant neoplasm of rectum - rectal ampulla  Differentiation:  Moderately differentiated</t>
         </is>
       </c>
       <c r="L2" s="30" t="inlineStr"/>
-      <c r="M2" s="30" t="inlineStr">
-        <is>
-          <t>Deficient</t>
-        </is>
-      </c>
-      <c r="N2" s="30" t="inlineStr"/>
+      <c r="M2" s="30" t="inlineStr"/>
+      <c r="N2" s="30" t="inlineStr">
+        <is>
+          <t>20/05/2025</t>
+        </is>
+      </c>
       <c r="O2" s="30" t="inlineStr"/>
       <c r="P2" s="30" t="inlineStr"/>
       <c r="Q2" s="30" t="inlineStr"/>
@@ -1313,7 +1309,7 @@
       <c r="S2" s="30" t="inlineStr"/>
       <c r="T2" s="30" t="inlineStr">
         <is>
-          <t>29/02/2025</t>
+          <t>26/05/1970</t>
         </is>
       </c>
       <c r="U2" s="30" t="inlineStr"/>
@@ -1326,7 +1322,11 @@
       </c>
       <c r="Y2" s="30" t="inlineStr"/>
       <c r="Z2" s="30" t="inlineStr"/>
-      <c r="AA2" s="30" t="inlineStr"/>
+      <c r="AA2" s="30" t="inlineStr">
+        <is>
+          <t>07/03/2025</t>
+        </is>
+      </c>
       <c r="AB2" s="30" t="inlineStr"/>
       <c r="AC2" s="30" t="inlineStr"/>
       <c r="AD2" s="30" t="inlineStr"/>
@@ -1346,7 +1346,11 @@
       <c r="AR2" s="30" t="inlineStr"/>
       <c r="AS2" s="30" t="inlineStr"/>
       <c r="AT2" s="30" t="inlineStr"/>
-      <c r="AU2" s="30" t="inlineStr"/>
+      <c r="AU2" s="30" t="inlineStr">
+        <is>
+          <t>29/02/2025</t>
+        </is>
+      </c>
       <c r="AV2" s="30" t="inlineStr"/>
       <c r="AW2" s="30" t="inlineStr"/>
       <c r="AX2" s="30" t="inlineStr"/>
@@ -1355,7 +1359,11 @@
       <c r="BA2" s="30" t="inlineStr"/>
       <c r="BB2" s="30" t="inlineStr"/>
       <c r="BC2" s="30" t="inlineStr"/>
-      <c r="BD2" s="30" t="inlineStr"/>
+      <c r="BD2" s="30" t="inlineStr">
+        <is>
+          <t>MRI Rectum, PET CT. Rediscuss at MDT for formal staging. Patient aware, decision RE treatment following further imaging and discussion.</t>
+        </is>
+      </c>
       <c r="BE2" s="30" t="inlineStr"/>
       <c r="BF2" s="30" t="inlineStr"/>
       <c r="BG2" s="30" t="inlineStr"/>
@@ -1414,16 +1422,8 @@
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr"/>
-      <c r="I3" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J3" s="30" t="inlineStr">
-        <is>
-          <t>polypoidal lesion in the low re</t>
-        </is>
-      </c>
+      <c r="I3" s="30" t="inlineStr"/>
+      <c r="J3" s="30" t="inlineStr"/>
       <c r="K3" s="30" t="inlineStr">
         <is>
           <t>ADENOCARCINOMA, NOT OTHERWISE SPECIFIED  ICD10 Code: 10 - C20: Malignant neoplasm of rectum - rectal ampulla  Differentiation:  Poorly differentiated</t>
@@ -1431,19 +1431,35 @@
       </c>
       <c r="L3" s="30" t="inlineStr"/>
       <c r="M3" s="30" t="inlineStr"/>
-      <c r="N3" s="30" t="inlineStr"/>
+      <c r="N3" s="30" t="inlineStr">
+        <is>
+          <t>22/2/2025</t>
+        </is>
+      </c>
       <c r="O3" s="30" t="inlineStr"/>
       <c r="P3" s="30" t="inlineStr"/>
-      <c r="Q3" s="30" t="inlineStr"/>
+      <c r="Q3" s="30" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
       <c r="R3" s="30" t="inlineStr"/>
       <c r="S3" s="30" t="inlineStr"/>
       <c r="T3" s="30" t="inlineStr">
         <is>
-          <t>22/2/2025</t>
-        </is>
-      </c>
-      <c r="U3" s="30" t="inlineStr"/>
-      <c r="V3" s="30" t="inlineStr"/>
+          <t>30/03/1944</t>
+        </is>
+      </c>
+      <c r="U3" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V3" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W3" s="30" t="inlineStr"/>
       <c r="X3" s="30" t="inlineStr">
         <is>
@@ -1452,7 +1468,11 @@
       </c>
       <c r="Y3" s="30" t="inlineStr"/>
       <c r="Z3" s="30" t="inlineStr"/>
-      <c r="AA3" s="30" t="inlineStr"/>
+      <c r="AA3" s="30" t="inlineStr">
+        <is>
+          <t>07/03/2025</t>
+        </is>
+      </c>
       <c r="AB3" s="30" t="inlineStr"/>
       <c r="AC3" s="30" t="inlineStr"/>
       <c r="AD3" s="30" t="inlineStr"/>
@@ -1528,7 +1548,11 @@
           <t>9990000003</t>
         </is>
       </c>
-      <c r="E4" s="30" t="inlineStr"/>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F4" s="30" t="inlineStr"/>
       <c r="G4" s="30" t="inlineStr"/>
       <c r="H4" s="30" t="inlineStr"/>
@@ -1541,20 +1565,36 @@
       </c>
       <c r="L4" s="30" t="inlineStr"/>
       <c r="M4" s="30" t="inlineStr"/>
-      <c r="N4" s="30" t="inlineStr"/>
+      <c r="N4" s="30" t="inlineStr">
+        <is>
+          <t>28/05/2025</t>
+        </is>
+      </c>
       <c r="O4" s="30" t="inlineStr"/>
       <c r="P4" s="30" t="inlineStr"/>
       <c r="Q4" s="30" t="inlineStr"/>
       <c r="R4" s="30" t="inlineStr"/>
       <c r="S4" s="30" t="inlineStr"/>
-      <c r="T4" s="30" t="inlineStr"/>
+      <c r="T4" s="30" t="inlineStr">
+        <is>
+          <t>19/12/1974</t>
+        </is>
+      </c>
       <c r="U4" s="30" t="inlineStr"/>
       <c r="V4" s="30" t="inlineStr"/>
       <c r="W4" s="30" t="inlineStr"/>
-      <c r="X4" s="30" t="inlineStr"/>
+      <c r="X4" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y4" s="30" t="inlineStr"/>
       <c r="Z4" s="30" t="inlineStr"/>
-      <c r="AA4" s="30" t="inlineStr"/>
+      <c r="AA4" s="30" t="inlineStr">
+        <is>
+          <t>07/03/2025</t>
+        </is>
+      </c>
       <c r="AB4" s="30" t="inlineStr"/>
       <c r="AC4" s="30" t="inlineStr"/>
       <c r="AD4" s="30" t="inlineStr"/>
@@ -1573,7 +1613,11 @@
       <c r="AQ4" s="30" t="inlineStr"/>
       <c r="AR4" s="30" t="inlineStr"/>
       <c r="AS4" s="30" t="inlineStr"/>
-      <c r="AT4" s="30" t="inlineStr"/>
+      <c r="AT4" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
       <c r="AU4" s="30" t="inlineStr"/>
       <c r="AV4" s="30" t="inlineStr"/>
       <c r="AW4" s="30" t="inlineStr"/>
@@ -1630,7 +1674,11 @@
           <t>9990000004</t>
         </is>
       </c>
-      <c r="E5" s="30" t="inlineStr"/>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F5" s="30" t="inlineStr"/>
       <c r="G5" s="30" t="inlineStr">
         <is>
@@ -1638,16 +1686,8 @@
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr"/>
-      <c r="I5" s="30" t="inlineStr">
-        <is>
-          <t>Flexi sig</t>
-        </is>
-      </c>
-      <c r="J5" s="30" t="inlineStr">
-        <is>
-          <t>scar seen  Outcome: to see surgeon, for</t>
-        </is>
-      </c>
+      <c r="I5" s="30" t="inlineStr"/>
+      <c r="J5" s="30" t="inlineStr"/>
       <c r="K5" s="30" t="inlineStr">
         <is>
           <t>ADENOCARCINOMA, NOT OTHERWISE SPECIFIED  ICD10 Code: 10 - C20: Malignant neoplasm of rectum - rectal ampulla  Differentiation:  Moderately differentiated</t>
@@ -1655,20 +1695,48 @@
       </c>
       <c r="L5" s="30" t="inlineStr"/>
       <c r="M5" s="30" t="inlineStr"/>
-      <c r="N5" s="30" t="inlineStr"/>
+      <c r="N5" s="30" t="inlineStr">
+        <is>
+          <t>06/05/2025</t>
+        </is>
+      </c>
       <c r="O5" s="30" t="inlineStr"/>
       <c r="P5" s="30" t="inlineStr"/>
       <c r="Q5" s="30" t="inlineStr"/>
-      <c r="R5" s="30" t="inlineStr"/>
+      <c r="R5" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S5" s="30" t="inlineStr"/>
-      <c r="T5" s="30" t="inlineStr"/>
-      <c r="U5" s="30" t="inlineStr"/>
-      <c r="V5" s="30" t="inlineStr"/>
+      <c r="T5" s="30" t="inlineStr">
+        <is>
+          <t>25/02/1943</t>
+        </is>
+      </c>
+      <c r="U5" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V5" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W5" s="30" t="inlineStr"/>
-      <c r="X5" s="30" t="inlineStr"/>
+      <c r="X5" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y5" s="30" t="inlineStr"/>
       <c r="Z5" s="30" t="inlineStr"/>
-      <c r="AA5" s="30" t="inlineStr"/>
+      <c r="AA5" s="30" t="inlineStr">
+        <is>
+          <t>13/09/2024</t>
+        </is>
+      </c>
       <c r="AB5" s="30" t="inlineStr"/>
       <c r="AC5" s="30" t="inlineStr"/>
       <c r="AD5" s="30" t="inlineStr"/>
@@ -1697,7 +1765,11 @@
       <c r="BA5" s="30" t="inlineStr"/>
       <c r="BB5" s="30" t="inlineStr"/>
       <c r="BC5" s="30" t="inlineStr"/>
-      <c r="BD5" s="30" t="inlineStr"/>
+      <c r="BD5" s="30" t="inlineStr">
+        <is>
+          <t>to see surgeon, for discussion with patient RE entering watch and wait</t>
+        </is>
+      </c>
       <c r="BE5" s="30" t="inlineStr"/>
       <c r="BF5" s="30" t="inlineStr"/>
       <c r="BG5" s="30" t="inlineStr"/>
@@ -1709,7 +1781,11 @@
       <c r="BM5" s="30" t="inlineStr"/>
       <c r="BN5" s="30" t="inlineStr"/>
       <c r="BO5" s="30" t="inlineStr"/>
-      <c r="BP5" s="30" t="inlineStr"/>
+      <c r="BP5" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="BQ5" s="30" t="inlineStr"/>
       <c r="BR5" s="30" t="inlineStr"/>
       <c r="BS5" s="30" t="inlineStr"/>
@@ -1744,7 +1820,11 @@
           <t>9998009005</t>
         </is>
       </c>
-      <c r="E6" s="30" t="inlineStr"/>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F6" s="30" t="inlineStr"/>
       <c r="G6" s="30" t="inlineStr"/>
       <c r="H6" s="30" t="inlineStr"/>
@@ -1757,20 +1837,36 @@
       </c>
       <c r="L6" s="30" t="inlineStr"/>
       <c r="M6" s="30" t="inlineStr"/>
-      <c r="N6" s="30" t="inlineStr"/>
+      <c r="N6" s="30" t="inlineStr">
+        <is>
+          <t>14/11/2024</t>
+        </is>
+      </c>
       <c r="O6" s="30" t="inlineStr"/>
       <c r="P6" s="30" t="inlineStr"/>
       <c r="Q6" s="30" t="inlineStr"/>
       <c r="R6" s="30" t="inlineStr"/>
       <c r="S6" s="30" t="inlineStr"/>
-      <c r="T6" s="30" t="inlineStr"/>
+      <c r="T6" s="30" t="inlineStr">
+        <is>
+          <t>16/11/1950</t>
+        </is>
+      </c>
       <c r="U6" s="30" t="inlineStr"/>
       <c r="V6" s="30" t="inlineStr"/>
       <c r="W6" s="30" t="inlineStr"/>
-      <c r="X6" s="30" t="inlineStr"/>
+      <c r="X6" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y6" s="30" t="inlineStr"/>
       <c r="Z6" s="30" t="inlineStr"/>
-      <c r="AA6" s="30" t="inlineStr"/>
+      <c r="AA6" s="30" t="inlineStr">
+        <is>
+          <t>14/11/2024</t>
+        </is>
+      </c>
       <c r="AB6" s="30" t="inlineStr"/>
       <c r="AC6" s="30" t="inlineStr"/>
       <c r="AD6" s="30" t="inlineStr"/>
@@ -1790,7 +1886,11 @@
       <c r="AR6" s="30" t="inlineStr"/>
       <c r="AS6" s="30" t="inlineStr"/>
       <c r="AT6" s="30" t="inlineStr"/>
-      <c r="AU6" s="30" t="inlineStr"/>
+      <c r="AU6" s="30" t="inlineStr">
+        <is>
+          <t>06/09/2024</t>
+        </is>
+      </c>
       <c r="AV6" s="30" t="inlineStr"/>
       <c r="AW6" s="30" t="inlineStr"/>
       <c r="AX6" s="30" t="inlineStr"/>
@@ -1846,7 +1946,11 @@
           <t>9998009006</t>
         </is>
       </c>
-      <c r="E7" s="30" t="inlineStr"/>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F7" s="30" t="inlineStr"/>
       <c r="G7" s="30" t="inlineStr"/>
       <c r="H7" s="30" t="inlineStr"/>
@@ -1859,20 +1963,48 @@
       </c>
       <c r="L7" s="30" t="inlineStr"/>
       <c r="M7" s="30" t="inlineStr"/>
-      <c r="N7" s="30" t="inlineStr"/>
+      <c r="N7" s="30" t="inlineStr">
+        <is>
+          <t>15/01/2025</t>
+        </is>
+      </c>
       <c r="O7" s="30" t="inlineStr"/>
       <c r="P7" s="30" t="inlineStr"/>
       <c r="Q7" s="30" t="inlineStr"/>
-      <c r="R7" s="30" t="inlineStr"/>
+      <c r="R7" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S7" s="30" t="inlineStr"/>
-      <c r="T7" s="30" t="inlineStr"/>
-      <c r="U7" s="30" t="inlineStr"/>
-      <c r="V7" s="30" t="inlineStr"/>
+      <c r="T7" s="30" t="inlineStr">
+        <is>
+          <t>18/08/1937</t>
+        </is>
+      </c>
+      <c r="U7" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V7" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W7" s="30" t="inlineStr"/>
-      <c r="X7" s="30" t="inlineStr"/>
+      <c r="X7" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y7" s="30" t="inlineStr"/>
       <c r="Z7" s="30" t="inlineStr"/>
-      <c r="AA7" s="30" t="inlineStr"/>
+      <c r="AA7" s="30" t="inlineStr">
+        <is>
+          <t>21/06/2024</t>
+        </is>
+      </c>
       <c r="AB7" s="30" t="inlineStr"/>
       <c r="AC7" s="30" t="inlineStr"/>
       <c r="AD7" s="30" t="inlineStr"/>
@@ -1892,7 +2024,11 @@
       <c r="AR7" s="30" t="inlineStr"/>
       <c r="AS7" s="30" t="inlineStr"/>
       <c r="AT7" s="30" t="inlineStr"/>
-      <c r="AU7" s="30" t="inlineStr"/>
+      <c r="AU7" s="30" t="inlineStr">
+        <is>
+          <t>31/10/2024</t>
+        </is>
+      </c>
       <c r="AV7" s="30" t="inlineStr"/>
       <c r="AW7" s="30" t="inlineStr"/>
       <c r="AX7" s="30" t="inlineStr"/>
@@ -1948,7 +2084,11 @@
           <t>9998009007</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr"/>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F8" s="30" t="inlineStr"/>
       <c r="G8" s="30" t="inlineStr"/>
       <c r="H8" s="30" t="inlineStr"/>
@@ -1961,20 +2101,36 @@
       </c>
       <c r="L8" s="30" t="inlineStr"/>
       <c r="M8" s="30" t="inlineStr"/>
-      <c r="N8" s="30" t="inlineStr"/>
+      <c r="N8" s="30" t="inlineStr">
+        <is>
+          <t>14/06/2024</t>
+        </is>
+      </c>
       <c r="O8" s="30" t="inlineStr"/>
       <c r="P8" s="30" t="inlineStr"/>
       <c r="Q8" s="30" t="inlineStr"/>
       <c r="R8" s="30" t="inlineStr"/>
       <c r="S8" s="30" t="inlineStr"/>
-      <c r="T8" s="30" t="inlineStr"/>
+      <c r="T8" s="30" t="inlineStr">
+        <is>
+          <t>27/12/1947</t>
+        </is>
+      </c>
       <c r="U8" s="30" t="inlineStr"/>
       <c r="V8" s="30" t="inlineStr"/>
       <c r="W8" s="30" t="inlineStr"/>
-      <c r="X8" s="30" t="inlineStr"/>
+      <c r="X8" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y8" s="30" t="inlineStr"/>
       <c r="Z8" s="30" t="inlineStr"/>
-      <c r="AA8" s="30" t="inlineStr"/>
+      <c r="AA8" s="30" t="inlineStr">
+        <is>
+          <t>20/08/2024</t>
+        </is>
+      </c>
       <c r="AB8" s="30" t="inlineStr"/>
       <c r="AC8" s="30" t="inlineStr"/>
       <c r="AD8" s="30" t="inlineStr"/>
@@ -2050,7 +2206,11 @@
           <t>9998009008</t>
         </is>
       </c>
-      <c r="E9" s="30" t="inlineStr"/>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F9" s="30" t="inlineStr"/>
       <c r="G9" s="30" t="inlineStr">
         <is>
@@ -2067,20 +2227,52 @@
       </c>
       <c r="L9" s="30" t="inlineStr"/>
       <c r="M9" s="30" t="inlineStr"/>
-      <c r="N9" s="30" t="inlineStr"/>
+      <c r="N9" s="30" t="inlineStr">
+        <is>
+          <t>21/10/2024</t>
+        </is>
+      </c>
       <c r="O9" s="30" t="inlineStr"/>
       <c r="P9" s="30" t="inlineStr"/>
-      <c r="Q9" s="30" t="inlineStr"/>
-      <c r="R9" s="30" t="inlineStr"/>
+      <c r="Q9" s="30" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="R9" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S9" s="30" t="inlineStr"/>
-      <c r="T9" s="30" t="inlineStr"/>
-      <c r="U9" s="30" t="inlineStr"/>
-      <c r="V9" s="30" t="inlineStr"/>
+      <c r="T9" s="30" t="inlineStr">
+        <is>
+          <t>08/08/1951</t>
+        </is>
+      </c>
+      <c r="U9" s="30" t="inlineStr">
+        <is>
+          <t>3a</t>
+        </is>
+      </c>
+      <c r="V9" s="30" t="inlineStr">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
       <c r="W9" s="30" t="inlineStr"/>
-      <c r="X9" s="30" t="inlineStr"/>
+      <c r="X9" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y9" s="30" t="inlineStr"/>
       <c r="Z9" s="30" t="inlineStr"/>
-      <c r="AA9" s="30" t="inlineStr"/>
+      <c r="AA9" s="30" t="inlineStr">
+        <is>
+          <t>10/04/2024</t>
+        </is>
+      </c>
       <c r="AB9" s="30" t="inlineStr"/>
       <c r="AC9" s="30" t="inlineStr"/>
       <c r="AD9" s="30" t="inlineStr"/>
@@ -2100,7 +2292,11 @@
       <c r="AR9" s="30" t="inlineStr"/>
       <c r="AS9" s="30" t="inlineStr"/>
       <c r="AT9" s="30" t="inlineStr"/>
-      <c r="AU9" s="30" t="inlineStr"/>
+      <c r="AU9" s="30" t="inlineStr">
+        <is>
+          <t>30/07/2024</t>
+        </is>
+      </c>
       <c r="AV9" s="30" t="inlineStr"/>
       <c r="AW9" s="30" t="inlineStr"/>
       <c r="AX9" s="30" t="inlineStr"/>
@@ -2156,7 +2352,11 @@
           <t>9998009009</t>
         </is>
       </c>
-      <c r="E10" s="30" t="inlineStr"/>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F10" s="30" t="inlineStr"/>
       <c r="G10" s="30" t="inlineStr">
         <is>
@@ -2173,20 +2373,36 @@
       </c>
       <c r="L10" s="30" t="inlineStr"/>
       <c r="M10" s="30" t="inlineStr"/>
-      <c r="N10" s="30" t="inlineStr"/>
+      <c r="N10" s="30" t="inlineStr">
+        <is>
+          <t>11/06/2024</t>
+        </is>
+      </c>
       <c r="O10" s="30" t="inlineStr"/>
       <c r="P10" s="30" t="inlineStr"/>
       <c r="Q10" s="30" t="inlineStr"/>
       <c r="R10" s="30" t="inlineStr"/>
       <c r="S10" s="30" t="inlineStr"/>
-      <c r="T10" s="30" t="inlineStr"/>
+      <c r="T10" s="30" t="inlineStr">
+        <is>
+          <t>18/03/1964</t>
+        </is>
+      </c>
       <c r="U10" s="30" t="inlineStr"/>
       <c r="V10" s="30" t="inlineStr"/>
       <c r="W10" s="30" t="inlineStr"/>
-      <c r="X10" s="30" t="inlineStr"/>
+      <c r="X10" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y10" s="30" t="inlineStr"/>
       <c r="Z10" s="30" t="inlineStr"/>
-      <c r="AA10" s="30" t="inlineStr"/>
+      <c r="AA10" s="30" t="inlineStr">
+        <is>
+          <t>18/09/2024</t>
+        </is>
+      </c>
       <c r="AB10" s="30" t="inlineStr"/>
       <c r="AC10" s="30" t="inlineStr"/>
       <c r="AD10" s="30" t="inlineStr"/>
@@ -2206,7 +2422,11 @@
       <c r="AR10" s="30" t="inlineStr"/>
       <c r="AS10" s="30" t="inlineStr"/>
       <c r="AT10" s="30" t="inlineStr"/>
-      <c r="AU10" s="30" t="inlineStr"/>
+      <c r="AU10" s="30" t="inlineStr">
+        <is>
+          <t>13/03/2024</t>
+        </is>
+      </c>
       <c r="AV10" s="30" t="inlineStr"/>
       <c r="AW10" s="30" t="inlineStr"/>
       <c r="AX10" s="30" t="inlineStr"/>
@@ -2262,7 +2482,11 @@
           <t>9998009010</t>
         </is>
       </c>
-      <c r="E11" s="30" t="inlineStr"/>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F11" s="30" t="inlineStr"/>
       <c r="G11" s="30" t="inlineStr"/>
       <c r="H11" s="30" t="inlineStr"/>
@@ -2275,20 +2499,48 @@
       </c>
       <c r="L11" s="30" t="inlineStr"/>
       <c r="M11" s="30" t="inlineStr"/>
-      <c r="N11" s="30" t="inlineStr"/>
+      <c r="N11" s="30" t="inlineStr">
+        <is>
+          <t>19/11/2024</t>
+        </is>
+      </c>
       <c r="O11" s="30" t="inlineStr"/>
       <c r="P11" s="30" t="inlineStr"/>
       <c r="Q11" s="30" t="inlineStr"/>
-      <c r="R11" s="30" t="inlineStr"/>
+      <c r="R11" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S11" s="30" t="inlineStr"/>
-      <c r="T11" s="30" t="inlineStr"/>
-      <c r="U11" s="30" t="inlineStr"/>
-      <c r="V11" s="30" t="inlineStr"/>
+      <c r="T11" s="30" t="inlineStr">
+        <is>
+          <t>20/06/1941</t>
+        </is>
+      </c>
+      <c r="U11" s="30" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="V11" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W11" s="30" t="inlineStr"/>
-      <c r="X11" s="30" t="inlineStr"/>
+      <c r="X11" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y11" s="30" t="inlineStr"/>
       <c r="Z11" s="30" t="inlineStr"/>
-      <c r="AA11" s="30" t="inlineStr"/>
+      <c r="AA11" s="30" t="inlineStr">
+        <is>
+          <t>19/02/2025</t>
+        </is>
+      </c>
       <c r="AB11" s="30" t="inlineStr"/>
       <c r="AC11" s="30" t="inlineStr"/>
       <c r="AD11" s="30" t="inlineStr"/>
@@ -2307,8 +2559,16 @@
       <c r="AQ11" s="30" t="inlineStr"/>
       <c r="AR11" s="30" t="inlineStr"/>
       <c r="AS11" s="30" t="inlineStr"/>
-      <c r="AT11" s="30" t="inlineStr"/>
-      <c r="AU11" s="30" t="inlineStr"/>
+      <c r="AT11" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
+      <c r="AU11" s="30" t="inlineStr">
+        <is>
+          <t>14/08/2024</t>
+        </is>
+      </c>
       <c r="AV11" s="30" t="inlineStr"/>
       <c r="AW11" s="30" t="inlineStr"/>
       <c r="AX11" s="30" t="inlineStr"/>
@@ -2364,7 +2624,11 @@
           <t>9998009011</t>
         </is>
       </c>
-      <c r="E12" s="30" t="inlineStr"/>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F12" s="30" t="inlineStr"/>
       <c r="G12" s="30" t="inlineStr"/>
       <c r="H12" s="30" t="inlineStr"/>
@@ -2377,20 +2641,36 @@
       </c>
       <c r="L12" s="30" t="inlineStr"/>
       <c r="M12" s="30" t="inlineStr"/>
-      <c r="N12" s="30" t="inlineStr"/>
+      <c r="N12" s="30" t="inlineStr">
+        <is>
+          <t>12/02/2025</t>
+        </is>
+      </c>
       <c r="O12" s="30" t="inlineStr"/>
       <c r="P12" s="30" t="inlineStr"/>
       <c r="Q12" s="30" t="inlineStr"/>
       <c r="R12" s="30" t="inlineStr"/>
       <c r="S12" s="30" t="inlineStr"/>
-      <c r="T12" s="30" t="inlineStr"/>
+      <c r="T12" s="30" t="inlineStr">
+        <is>
+          <t>24/03/1957</t>
+        </is>
+      </c>
       <c r="U12" s="30" t="inlineStr"/>
       <c r="V12" s="30" t="inlineStr"/>
       <c r="W12" s="30" t="inlineStr"/>
-      <c r="X12" s="30" t="inlineStr"/>
+      <c r="X12" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y12" s="30" t="inlineStr"/>
       <c r="Z12" s="30" t="inlineStr"/>
-      <c r="AA12" s="30" t="inlineStr"/>
+      <c r="AA12" s="30" t="inlineStr">
+        <is>
+          <t>18/05/2024</t>
+        </is>
+      </c>
       <c r="AB12" s="30" t="inlineStr"/>
       <c r="AC12" s="30" t="inlineStr"/>
       <c r="AD12" s="30" t="inlineStr"/>
@@ -2466,7 +2746,11 @@
           <t>9998009012</t>
         </is>
       </c>
-      <c r="E13" s="30" t="inlineStr"/>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F13" s="30" t="inlineStr"/>
       <c r="G13" s="30" t="inlineStr"/>
       <c r="H13" s="30" t="inlineStr"/>
@@ -2479,20 +2763,44 @@
       </c>
       <c r="L13" s="30" t="inlineStr"/>
       <c r="M13" s="30" t="inlineStr"/>
-      <c r="N13" s="30" t="inlineStr"/>
+      <c r="N13" s="30" t="inlineStr">
+        <is>
+          <t>19/07/2024</t>
+        </is>
+      </c>
       <c r="O13" s="30" t="inlineStr"/>
       <c r="P13" s="30" t="inlineStr"/>
       <c r="Q13" s="30" t="inlineStr"/>
       <c r="R13" s="30" t="inlineStr"/>
       <c r="S13" s="30" t="inlineStr"/>
-      <c r="T13" s="30" t="inlineStr"/>
-      <c r="U13" s="30" t="inlineStr"/>
-      <c r="V13" s="30" t="inlineStr"/>
+      <c r="T13" s="30" t="inlineStr">
+        <is>
+          <t>22/10/1958</t>
+        </is>
+      </c>
+      <c r="U13" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V13" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W13" s="30" t="inlineStr"/>
-      <c r="X13" s="30" t="inlineStr"/>
+      <c r="X13" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y13" s="30" t="inlineStr"/>
       <c r="Z13" s="30" t="inlineStr"/>
-      <c r="AA13" s="30" t="inlineStr"/>
+      <c r="AA13" s="30" t="inlineStr">
+        <is>
+          <t>12/01/2025</t>
+        </is>
+      </c>
       <c r="AB13" s="30" t="inlineStr"/>
       <c r="AC13" s="30" t="inlineStr"/>
       <c r="AD13" s="30" t="inlineStr"/>
@@ -2511,8 +2819,16 @@
       <c r="AQ13" s="30" t="inlineStr"/>
       <c r="AR13" s="30" t="inlineStr"/>
       <c r="AS13" s="30" t="inlineStr"/>
-      <c r="AT13" s="30" t="inlineStr"/>
-      <c r="AU13" s="30" t="inlineStr"/>
+      <c r="AT13" s="30" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="AU13" s="30" t="inlineStr">
+        <is>
+          <t>11/05/2024</t>
+        </is>
+      </c>
       <c r="AV13" s="30" t="inlineStr"/>
       <c r="AW13" s="30" t="inlineStr"/>
       <c r="AX13" s="30" t="inlineStr"/>
@@ -2568,7 +2884,11 @@
           <t>9998009013</t>
         </is>
       </c>
-      <c r="E14" s="30" t="inlineStr"/>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F14" s="30" t="inlineStr"/>
       <c r="G14" s="30" t="inlineStr"/>
       <c r="H14" s="30" t="inlineStr"/>
@@ -2581,22 +2901,42 @@
       </c>
       <c r="L14" s="30" t="inlineStr"/>
       <c r="M14" s="30" t="inlineStr"/>
-      <c r="N14" s="30" t="inlineStr"/>
+      <c r="N14" s="30" t="inlineStr">
+        <is>
+          <t>15/03/2025</t>
+        </is>
+      </c>
       <c r="O14" s="30" t="inlineStr"/>
       <c r="P14" s="30" t="inlineStr"/>
       <c r="Q14" s="30" t="inlineStr"/>
       <c r="R14" s="30" t="inlineStr"/>
       <c r="S14" s="30" t="inlineStr"/>
-      <c r="T14" s="30" t="inlineStr"/>
+      <c r="T14" s="30" t="inlineStr">
+        <is>
+          <t>28/04/1952</t>
+        </is>
+      </c>
       <c r="U14" s="30" t="inlineStr"/>
       <c r="V14" s="30" t="inlineStr"/>
       <c r="W14" s="30" t="inlineStr"/>
-      <c r="X14" s="30" t="inlineStr"/>
+      <c r="X14" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y14" s="30" t="inlineStr"/>
       <c r="Z14" s="30" t="inlineStr"/>
-      <c r="AA14" s="30" t="inlineStr"/>
+      <c r="AA14" s="30" t="inlineStr">
+        <is>
+          <t>27/02/2024</t>
+        </is>
+      </c>
       <c r="AB14" s="30" t="inlineStr"/>
-      <c r="AC14" s="30" t="inlineStr"/>
+      <c r="AC14" s="30" t="inlineStr">
+        <is>
+          <t>curative</t>
+        </is>
+      </c>
       <c r="AD14" s="30" t="inlineStr"/>
       <c r="AE14" s="30" t="inlineStr"/>
       <c r="AF14" s="30" t="inlineStr"/>
@@ -2613,8 +2953,16 @@
       <c r="AQ14" s="30" t="inlineStr"/>
       <c r="AR14" s="30" t="inlineStr"/>
       <c r="AS14" s="30" t="inlineStr"/>
-      <c r="AT14" s="30" t="inlineStr"/>
-      <c r="AU14" s="30" t="inlineStr"/>
+      <c r="AT14" s="30" t="inlineStr">
+        <is>
+          <t>curative</t>
+        </is>
+      </c>
+      <c r="AU14" s="30" t="inlineStr">
+        <is>
+          <t>29/12/2024</t>
+        </is>
+      </c>
       <c r="AV14" s="30" t="inlineStr"/>
       <c r="AW14" s="30" t="inlineStr"/>
       <c r="AX14" s="30" t="inlineStr"/>
@@ -2670,7 +3018,11 @@
           <t>9998009014</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr"/>
+      <c r="E15" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F15" s="30" t="inlineStr"/>
       <c r="G15" s="30" t="inlineStr"/>
       <c r="H15" s="30" t="inlineStr"/>
@@ -2683,20 +3035,48 @@
       </c>
       <c r="L15" s="30" t="inlineStr"/>
       <c r="M15" s="30" t="inlineStr"/>
-      <c r="N15" s="30" t="inlineStr"/>
+      <c r="N15" s="30" t="inlineStr">
+        <is>
+          <t>29/04/2024</t>
+        </is>
+      </c>
       <c r="O15" s="30" t="inlineStr"/>
       <c r="P15" s="30" t="inlineStr"/>
       <c r="Q15" s="30" t="inlineStr"/>
-      <c r="R15" s="30" t="inlineStr"/>
+      <c r="R15" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S15" s="30" t="inlineStr"/>
-      <c r="T15" s="30" t="inlineStr"/>
-      <c r="U15" s="30" t="inlineStr"/>
-      <c r="V15" s="30" t="inlineStr"/>
+      <c r="T15" s="30" t="inlineStr">
+        <is>
+          <t>20/06/1964</t>
+        </is>
+      </c>
+      <c r="U15" s="30" t="inlineStr">
+        <is>
+          <t>3c</t>
+        </is>
+      </c>
+      <c r="V15" s="30" t="inlineStr">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
       <c r="W15" s="30" t="inlineStr"/>
-      <c r="X15" s="30" t="inlineStr"/>
+      <c r="X15" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y15" s="30" t="inlineStr"/>
       <c r="Z15" s="30" t="inlineStr"/>
-      <c r="AA15" s="30" t="inlineStr"/>
+      <c r="AA15" s="30" t="inlineStr">
+        <is>
+          <t>05/01/2025</t>
+        </is>
+      </c>
       <c r="AB15" s="30" t="inlineStr"/>
       <c r="AC15" s="30" t="inlineStr"/>
       <c r="AD15" s="30" t="inlineStr"/>
@@ -2772,7 +3152,11 @@
           <t>9998009015</t>
         </is>
       </c>
-      <c r="E16" s="30" t="inlineStr"/>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F16" s="30" t="inlineStr"/>
       <c r="G16" s="30" t="inlineStr">
         <is>
@@ -2789,20 +3173,44 @@
       </c>
       <c r="L16" s="30" t="inlineStr"/>
       <c r="M16" s="30" t="inlineStr"/>
-      <c r="N16" s="30" t="inlineStr"/>
+      <c r="N16" s="30" t="inlineStr">
+        <is>
+          <t>08/03/2025</t>
+        </is>
+      </c>
       <c r="O16" s="30" t="inlineStr"/>
       <c r="P16" s="30" t="inlineStr"/>
-      <c r="Q16" s="30" t="inlineStr"/>
+      <c r="Q16" s="30" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
       <c r="R16" s="30" t="inlineStr"/>
       <c r="S16" s="30" t="inlineStr"/>
-      <c r="T16" s="30" t="inlineStr"/>
-      <c r="U16" s="30" t="inlineStr"/>
+      <c r="T16" s="30" t="inlineStr">
+        <is>
+          <t>27/03/1972</t>
+        </is>
+      </c>
+      <c r="U16" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="V16" s="30" t="inlineStr"/>
       <c r="W16" s="30" t="inlineStr"/>
-      <c r="X16" s="30" t="inlineStr"/>
+      <c r="X16" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y16" s="30" t="inlineStr"/>
       <c r="Z16" s="30" t="inlineStr"/>
-      <c r="AA16" s="30" t="inlineStr"/>
+      <c r="AA16" s="30" t="inlineStr">
+        <is>
+          <t>01/12/2024</t>
+        </is>
+      </c>
       <c r="AB16" s="30" t="inlineStr"/>
       <c r="AC16" s="30" t="inlineStr"/>
       <c r="AD16" s="30" t="inlineStr"/>
@@ -2878,7 +3286,11 @@
           <t>9998009016</t>
         </is>
       </c>
-      <c r="E17" s="30" t="inlineStr"/>
+      <c r="E17" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F17" s="30" t="inlineStr"/>
       <c r="G17" s="30" t="inlineStr"/>
       <c r="H17" s="30" t="inlineStr"/>
@@ -2891,20 +3303,44 @@
       </c>
       <c r="L17" s="30" t="inlineStr"/>
       <c r="M17" s="30" t="inlineStr"/>
-      <c r="N17" s="30" t="inlineStr"/>
+      <c r="N17" s="30" t="inlineStr">
+        <is>
+          <t>13/01/2025</t>
+        </is>
+      </c>
       <c r="O17" s="30" t="inlineStr"/>
       <c r="P17" s="30" t="inlineStr"/>
       <c r="Q17" s="30" t="inlineStr"/>
       <c r="R17" s="30" t="inlineStr"/>
       <c r="S17" s="30" t="inlineStr"/>
-      <c r="T17" s="30" t="inlineStr"/>
-      <c r="U17" s="30" t="inlineStr"/>
-      <c r="V17" s="30" t="inlineStr"/>
+      <c r="T17" s="30" t="inlineStr">
+        <is>
+          <t>03/03/1984</t>
+        </is>
+      </c>
+      <c r="U17" s="30" t="inlineStr">
+        <is>
+          <t>3d</t>
+        </is>
+      </c>
+      <c r="V17" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W17" s="30" t="inlineStr"/>
-      <c r="X17" s="30" t="inlineStr"/>
+      <c r="X17" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y17" s="30" t="inlineStr"/>
       <c r="Z17" s="30" t="inlineStr"/>
-      <c r="AA17" s="30" t="inlineStr"/>
+      <c r="AA17" s="30" t="inlineStr">
+        <is>
+          <t>21/09/2024</t>
+        </is>
+      </c>
       <c r="AB17" s="30" t="inlineStr"/>
       <c r="AC17" s="30" t="inlineStr"/>
       <c r="AD17" s="30" t="inlineStr"/>
@@ -2980,7 +3416,11 @@
           <t>9998009017</t>
         </is>
       </c>
-      <c r="E18" s="30" t="inlineStr"/>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F18" s="30" t="inlineStr"/>
       <c r="G18" s="30" t="inlineStr"/>
       <c r="H18" s="30" t="inlineStr"/>
@@ -2993,20 +3433,36 @@
       </c>
       <c r="L18" s="30" t="inlineStr"/>
       <c r="M18" s="30" t="inlineStr"/>
-      <c r="N18" s="30" t="inlineStr"/>
+      <c r="N18" s="30" t="inlineStr">
+        <is>
+          <t>14/09/2024</t>
+        </is>
+      </c>
       <c r="O18" s="30" t="inlineStr"/>
       <c r="P18" s="30" t="inlineStr"/>
       <c r="Q18" s="30" t="inlineStr"/>
       <c r="R18" s="30" t="inlineStr"/>
       <c r="S18" s="30" t="inlineStr"/>
-      <c r="T18" s="30" t="inlineStr"/>
+      <c r="T18" s="30" t="inlineStr">
+        <is>
+          <t>25/07/1965</t>
+        </is>
+      </c>
       <c r="U18" s="30" t="inlineStr"/>
       <c r="V18" s="30" t="inlineStr"/>
       <c r="W18" s="30" t="inlineStr"/>
-      <c r="X18" s="30" t="inlineStr"/>
+      <c r="X18" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y18" s="30" t="inlineStr"/>
       <c r="Z18" s="30" t="inlineStr"/>
-      <c r="AA18" s="30" t="inlineStr"/>
+      <c r="AA18" s="30" t="inlineStr">
+        <is>
+          <t>20/10/2024</t>
+        </is>
+      </c>
       <c r="AB18" s="30" t="inlineStr"/>
       <c r="AC18" s="30" t="inlineStr"/>
       <c r="AD18" s="30" t="inlineStr"/>
@@ -3082,7 +3538,11 @@
           <t>9998009018</t>
         </is>
       </c>
-      <c r="E19" s="30" t="inlineStr"/>
+      <c r="E19" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F19" s="30" t="inlineStr"/>
       <c r="G19" s="30" t="inlineStr"/>
       <c r="H19" s="30" t="inlineStr"/>
@@ -3095,20 +3555,36 @@
       </c>
       <c r="L19" s="30" t="inlineStr"/>
       <c r="M19" s="30" t="inlineStr"/>
-      <c r="N19" s="30" t="inlineStr"/>
+      <c r="N19" s="30" t="inlineStr">
+        <is>
+          <t>21/12/2024</t>
+        </is>
+      </c>
       <c r="O19" s="30" t="inlineStr"/>
       <c r="P19" s="30" t="inlineStr"/>
       <c r="Q19" s="30" t="inlineStr"/>
       <c r="R19" s="30" t="inlineStr"/>
       <c r="S19" s="30" t="inlineStr"/>
-      <c r="T19" s="30" t="inlineStr"/>
+      <c r="T19" s="30" t="inlineStr">
+        <is>
+          <t>28/10/1981</t>
+        </is>
+      </c>
       <c r="U19" s="30" t="inlineStr"/>
       <c r="V19" s="30" t="inlineStr"/>
       <c r="W19" s="30" t="inlineStr"/>
-      <c r="X19" s="30" t="inlineStr"/>
+      <c r="X19" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y19" s="30" t="inlineStr"/>
       <c r="Z19" s="30" t="inlineStr"/>
-      <c r="AA19" s="30" t="inlineStr"/>
+      <c r="AA19" s="30" t="inlineStr">
+        <is>
+          <t>30/01/2024</t>
+        </is>
+      </c>
       <c r="AB19" s="30" t="inlineStr"/>
       <c r="AC19" s="30" t="inlineStr"/>
       <c r="AD19" s="30" t="inlineStr"/>
@@ -3128,7 +3604,11 @@
       <c r="AR19" s="30" t="inlineStr"/>
       <c r="AS19" s="30" t="inlineStr"/>
       <c r="AT19" s="30" t="inlineStr"/>
-      <c r="AU19" s="30" t="inlineStr"/>
+      <c r="AU19" s="30" t="inlineStr">
+        <is>
+          <t>29/09/2024</t>
+        </is>
+      </c>
       <c r="AV19" s="30" t="inlineStr"/>
       <c r="AW19" s="30" t="inlineStr"/>
       <c r="AX19" s="30" t="inlineStr"/>
@@ -3184,7 +3664,11 @@
           <t>9990000019</t>
         </is>
       </c>
-      <c r="E20" s="30" t="inlineStr"/>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F20" s="30" t="inlineStr"/>
       <c r="G20" s="30" t="inlineStr"/>
       <c r="H20" s="30" t="inlineStr"/>
@@ -3197,20 +3681,44 @@
       </c>
       <c r="L20" s="30" t="inlineStr"/>
       <c r="M20" s="30" t="inlineStr"/>
-      <c r="N20" s="30" t="inlineStr"/>
+      <c r="N20" s="30" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
       <c r="O20" s="30" t="inlineStr"/>
       <c r="P20" s="30" t="inlineStr"/>
       <c r="Q20" s="30" t="inlineStr"/>
       <c r="R20" s="30" t="inlineStr"/>
       <c r="S20" s="30" t="inlineStr"/>
-      <c r="T20" s="30" t="inlineStr"/>
-      <c r="U20" s="30" t="inlineStr"/>
-      <c r="V20" s="30" t="inlineStr"/>
+      <c r="T20" s="30" t="inlineStr">
+        <is>
+          <t>17/05/1940</t>
+        </is>
+      </c>
+      <c r="U20" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V20" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W20" s="30" t="inlineStr"/>
-      <c r="X20" s="30" t="inlineStr"/>
+      <c r="X20" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y20" s="30" t="inlineStr"/>
       <c r="Z20" s="30" t="inlineStr"/>
-      <c r="AA20" s="30" t="inlineStr"/>
+      <c r="AA20" s="30" t="inlineStr">
+        <is>
+          <t>02/01/2024</t>
+        </is>
+      </c>
       <c r="AB20" s="30" t="inlineStr"/>
       <c r="AC20" s="30" t="inlineStr"/>
       <c r="AD20" s="30" t="inlineStr"/>
@@ -3286,7 +3794,11 @@
           <t>9990000020</t>
         </is>
       </c>
-      <c r="E21" s="30" t="inlineStr"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="inlineStr"/>
       <c r="G21" s="30" t="inlineStr"/>
       <c r="H21" s="30" t="inlineStr"/>
@@ -3299,20 +3811,36 @@
       </c>
       <c r="L21" s="30" t="inlineStr"/>
       <c r="M21" s="30" t="inlineStr"/>
-      <c r="N21" s="30" t="inlineStr"/>
+      <c r="N21" s="30" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
       <c r="O21" s="30" t="inlineStr"/>
       <c r="P21" s="30" t="inlineStr"/>
       <c r="Q21" s="30" t="inlineStr"/>
       <c r="R21" s="30" t="inlineStr"/>
       <c r="S21" s="30" t="inlineStr"/>
-      <c r="T21" s="30" t="inlineStr"/>
+      <c r="T21" s="30" t="inlineStr">
+        <is>
+          <t>03/07/1979</t>
+        </is>
+      </c>
       <c r="U21" s="30" t="inlineStr"/>
       <c r="V21" s="30" t="inlineStr"/>
       <c r="W21" s="30" t="inlineStr"/>
-      <c r="X21" s="30" t="inlineStr"/>
+      <c r="X21" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y21" s="30" t="inlineStr"/>
       <c r="Z21" s="30" t="inlineStr"/>
-      <c r="AA21" s="30" t="inlineStr"/>
+      <c r="AA21" s="30" t="inlineStr">
+        <is>
+          <t>07/03/2025</t>
+        </is>
+      </c>
       <c r="AB21" s="30" t="inlineStr"/>
       <c r="AC21" s="30" t="inlineStr"/>
       <c r="AD21" s="30" t="inlineStr"/>
@@ -3331,7 +3859,11 @@
       <c r="AQ21" s="30" t="inlineStr"/>
       <c r="AR21" s="30" t="inlineStr"/>
       <c r="AS21" s="30" t="inlineStr"/>
-      <c r="AT21" s="30" t="inlineStr"/>
+      <c r="AT21" s="30" t="inlineStr">
+        <is>
+          <t>hemicolectomy</t>
+        </is>
+      </c>
       <c r="AU21" s="30" t="inlineStr"/>
       <c r="AV21" s="30" t="inlineStr"/>
       <c r="AW21" s="30" t="inlineStr"/>
@@ -3388,7 +3920,11 @@
           <t>9990000021</t>
         </is>
       </c>
-      <c r="E22" s="30" t="inlineStr"/>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F22" s="30" t="inlineStr"/>
       <c r="G22" s="30" t="inlineStr"/>
       <c r="H22" s="30" t="inlineStr"/>
@@ -3401,20 +3937,36 @@
       </c>
       <c r="L22" s="30" t="inlineStr"/>
       <c r="M22" s="30" t="inlineStr"/>
-      <c r="N22" s="30" t="inlineStr"/>
+      <c r="N22" s="30" t="inlineStr">
+        <is>
+          <t>08/05/2025</t>
+        </is>
+      </c>
       <c r="O22" s="30" t="inlineStr"/>
       <c r="P22" s="30" t="inlineStr"/>
       <c r="Q22" s="30" t="inlineStr"/>
       <c r="R22" s="30" t="inlineStr"/>
       <c r="S22" s="30" t="inlineStr"/>
-      <c r="T22" s="30" t="inlineStr"/>
+      <c r="T22" s="30" t="inlineStr">
+        <is>
+          <t>02/02/1939</t>
+        </is>
+      </c>
       <c r="U22" s="30" t="inlineStr"/>
       <c r="V22" s="30" t="inlineStr"/>
       <c r="W22" s="30" t="inlineStr"/>
-      <c r="X22" s="30" t="inlineStr"/>
+      <c r="X22" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y22" s="30" t="inlineStr"/>
       <c r="Z22" s="30" t="inlineStr"/>
-      <c r="AA22" s="30" t="inlineStr"/>
+      <c r="AA22" s="30" t="inlineStr">
+        <is>
+          <t>28/02/2025</t>
+        </is>
+      </c>
       <c r="AB22" s="30" t="inlineStr"/>
       <c r="AC22" s="30" t="inlineStr"/>
       <c r="AD22" s="30" t="inlineStr"/>
@@ -3434,7 +3986,11 @@
       <c r="AR22" s="30" t="inlineStr"/>
       <c r="AS22" s="30" t="inlineStr"/>
       <c r="AT22" s="30" t="inlineStr"/>
-      <c r="AU22" s="30" t="inlineStr"/>
+      <c r="AU22" s="30" t="inlineStr">
+        <is>
+          <t>07/02/2025</t>
+        </is>
+      </c>
       <c r="AV22" s="30" t="inlineStr"/>
       <c r="AW22" s="30" t="inlineStr"/>
       <c r="AX22" s="30" t="inlineStr"/>
@@ -3490,7 +4046,11 @@
           <t>9990000022</t>
         </is>
       </c>
-      <c r="E23" s="30" t="inlineStr"/>
+      <c r="E23" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F23" s="30" t="inlineStr"/>
       <c r="G23" s="30" t="inlineStr">
         <is>
@@ -3507,20 +4067,44 @@
       </c>
       <c r="L23" s="30" t="inlineStr"/>
       <c r="M23" s="30" t="inlineStr"/>
-      <c r="N23" s="30" t="inlineStr"/>
+      <c r="N23" s="30" t="inlineStr">
+        <is>
+          <t>24/01/2025</t>
+        </is>
+      </c>
       <c r="O23" s="30" t="inlineStr"/>
       <c r="P23" s="30" t="inlineStr"/>
       <c r="Q23" s="30" t="inlineStr"/>
       <c r="R23" s="30" t="inlineStr"/>
       <c r="S23" s="30" t="inlineStr"/>
-      <c r="T23" s="30" t="inlineStr"/>
-      <c r="U23" s="30" t="inlineStr"/>
-      <c r="V23" s="30" t="inlineStr"/>
+      <c r="T23" s="30" t="inlineStr">
+        <is>
+          <t>20/05/1971</t>
+        </is>
+      </c>
+      <c r="U23" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V23" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W23" s="30" t="inlineStr"/>
-      <c r="X23" s="30" t="inlineStr"/>
+      <c r="X23" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y23" s="30" t="inlineStr"/>
       <c r="Z23" s="30" t="inlineStr"/>
-      <c r="AA23" s="30" t="inlineStr"/>
+      <c r="AA23" s="30" t="inlineStr">
+        <is>
+          <t>26/07/2024</t>
+        </is>
+      </c>
       <c r="AB23" s="30" t="inlineStr"/>
       <c r="AC23" s="30" t="inlineStr"/>
       <c r="AD23" s="30" t="inlineStr"/>
@@ -3539,7 +4123,11 @@
       <c r="AQ23" s="30" t="inlineStr"/>
       <c r="AR23" s="30" t="inlineStr"/>
       <c r="AS23" s="30" t="inlineStr"/>
-      <c r="AT23" s="30" t="inlineStr"/>
+      <c r="AT23" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
       <c r="AU23" s="30" t="inlineStr"/>
       <c r="AV23" s="30" t="inlineStr"/>
       <c r="AW23" s="30" t="inlineStr"/>
@@ -3596,7 +4184,11 @@
           <t>9990000023</t>
         </is>
       </c>
-      <c r="E24" s="30" t="inlineStr"/>
+      <c r="E24" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F24" s="30" t="inlineStr"/>
       <c r="G24" s="30" t="inlineStr">
         <is>
@@ -3613,20 +4205,36 @@
       </c>
       <c r="L24" s="30" t="inlineStr"/>
       <c r="M24" s="30" t="inlineStr"/>
-      <c r="N24" s="30" t="inlineStr"/>
+      <c r="N24" s="30" t="inlineStr">
+        <is>
+          <t>12/07/2024</t>
+        </is>
+      </c>
       <c r="O24" s="30" t="inlineStr"/>
       <c r="P24" s="30" t="inlineStr"/>
       <c r="Q24" s="30" t="inlineStr"/>
       <c r="R24" s="30" t="inlineStr"/>
       <c r="S24" s="30" t="inlineStr"/>
-      <c r="T24" s="30" t="inlineStr"/>
+      <c r="T24" s="30" t="inlineStr">
+        <is>
+          <t>18/06/1941</t>
+        </is>
+      </c>
       <c r="U24" s="30" t="inlineStr"/>
       <c r="V24" s="30" t="inlineStr"/>
       <c r="W24" s="30" t="inlineStr"/>
-      <c r="X24" s="30" t="inlineStr"/>
+      <c r="X24" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y24" s="30" t="inlineStr"/>
       <c r="Z24" s="30" t="inlineStr"/>
-      <c r="AA24" s="30" t="inlineStr"/>
+      <c r="AA24" s="30" t="inlineStr">
+        <is>
+          <t>10/01/2025</t>
+        </is>
+      </c>
       <c r="AB24" s="30" t="inlineStr"/>
       <c r="AC24" s="30" t="inlineStr"/>
       <c r="AD24" s="30" t="inlineStr"/>
@@ -3702,7 +4310,11 @@
           <t>9990000024</t>
         </is>
       </c>
-      <c r="E25" s="30" t="inlineStr"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="inlineStr"/>
       <c r="G25" s="30" t="inlineStr"/>
       <c r="H25" s="30" t="inlineStr"/>
@@ -3715,20 +4327,44 @@
       </c>
       <c r="L25" s="30" t="inlineStr"/>
       <c r="M25" s="30" t="inlineStr"/>
-      <c r="N25" s="30" t="inlineStr"/>
+      <c r="N25" s="30" t="inlineStr">
+        <is>
+          <t>13/03/2025</t>
+        </is>
+      </c>
       <c r="O25" s="30" t="inlineStr"/>
       <c r="P25" s="30" t="inlineStr"/>
       <c r="Q25" s="30" t="inlineStr"/>
       <c r="R25" s="30" t="inlineStr"/>
       <c r="S25" s="30" t="inlineStr"/>
-      <c r="T25" s="30" t="inlineStr"/>
-      <c r="U25" s="30" t="inlineStr"/>
-      <c r="V25" s="30" t="inlineStr"/>
+      <c r="T25" s="30" t="inlineStr">
+        <is>
+          <t>06/01/1963</t>
+        </is>
+      </c>
+      <c r="U25" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V25" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W25" s="30" t="inlineStr"/>
-      <c r="X25" s="30" t="inlineStr"/>
+      <c r="X25" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y25" s="30" t="inlineStr"/>
       <c r="Z25" s="30" t="inlineStr"/>
-      <c r="AA25" s="30" t="inlineStr"/>
+      <c r="AA25" s="30" t="inlineStr">
+        <is>
+          <t>07/02/2024</t>
+        </is>
+      </c>
       <c r="AB25" s="30" t="inlineStr"/>
       <c r="AC25" s="30" t="inlineStr"/>
       <c r="AD25" s="30" t="inlineStr"/>
@@ -3747,8 +4383,16 @@
       <c r="AQ25" s="30" t="inlineStr"/>
       <c r="AR25" s="30" t="inlineStr"/>
       <c r="AS25" s="30" t="inlineStr"/>
-      <c r="AT25" s="30" t="inlineStr"/>
-      <c r="AU25" s="30" t="inlineStr"/>
+      <c r="AT25" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
+      <c r="AU25" s="30" t="inlineStr">
+        <is>
+          <t>03/01/2025</t>
+        </is>
+      </c>
       <c r="AV25" s="30" t="inlineStr"/>
       <c r="AW25" s="30" t="inlineStr"/>
       <c r="AX25" s="30" t="inlineStr"/>
@@ -3804,7 +4448,11 @@
           <t>9990000025</t>
         </is>
       </c>
-      <c r="E26" s="30" t="inlineStr"/>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F26" s="30" t="inlineStr"/>
       <c r="G26" s="30" t="inlineStr"/>
       <c r="H26" s="30" t="inlineStr"/>
@@ -3817,20 +4465,48 @@
       </c>
       <c r="L26" s="30" t="inlineStr"/>
       <c r="M26" s="30" t="inlineStr"/>
-      <c r="N26" s="30" t="inlineStr"/>
+      <c r="N26" s="30" t="inlineStr">
+        <is>
+          <t>09/04/2024</t>
+        </is>
+      </c>
       <c r="O26" s="30" t="inlineStr"/>
       <c r="P26" s="30" t="inlineStr"/>
-      <c r="Q26" s="30" t="inlineStr"/>
-      <c r="R26" s="30" t="inlineStr"/>
+      <c r="Q26" s="30" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="R26" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S26" s="30" t="inlineStr"/>
-      <c r="T26" s="30" t="inlineStr"/>
-      <c r="U26" s="30" t="inlineStr"/>
+      <c r="T26" s="30" t="inlineStr">
+        <is>
+          <t>20/09/1957</t>
+        </is>
+      </c>
+      <c r="U26" s="30" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
       <c r="V26" s="30" t="inlineStr"/>
       <c r="W26" s="30" t="inlineStr"/>
-      <c r="X26" s="30" t="inlineStr"/>
+      <c r="X26" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y26" s="30" t="inlineStr"/>
       <c r="Z26" s="30" t="inlineStr"/>
-      <c r="AA26" s="30" t="inlineStr"/>
+      <c r="AA26" s="30" t="inlineStr">
+        <is>
+          <t>30/07/2024</t>
+        </is>
+      </c>
       <c r="AB26" s="30" t="inlineStr"/>
       <c r="AC26" s="30" t="inlineStr"/>
       <c r="AD26" s="30" t="inlineStr"/>
@@ -3850,7 +4526,11 @@
       <c r="AR26" s="30" t="inlineStr"/>
       <c r="AS26" s="30" t="inlineStr"/>
       <c r="AT26" s="30" t="inlineStr"/>
-      <c r="AU26" s="30" t="inlineStr"/>
+      <c r="AU26" s="30" t="inlineStr">
+        <is>
+          <t>24/01/2024</t>
+        </is>
+      </c>
       <c r="AV26" s="30" t="inlineStr"/>
       <c r="AW26" s="30" t="inlineStr"/>
       <c r="AX26" s="30" t="inlineStr"/>
@@ -3906,7 +4586,11 @@
           <t>9990000026</t>
         </is>
       </c>
-      <c r="E27" s="30" t="inlineStr"/>
+      <c r="E27" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F27" s="30" t="inlineStr"/>
       <c r="G27" s="30" t="inlineStr">
         <is>
@@ -3923,20 +4607,36 @@
       </c>
       <c r="L27" s="30" t="inlineStr"/>
       <c r="M27" s="30" t="inlineStr"/>
-      <c r="N27" s="30" t="inlineStr"/>
+      <c r="N27" s="30" t="inlineStr">
+        <is>
+          <t>23/07/2024</t>
+        </is>
+      </c>
       <c r="O27" s="30" t="inlineStr"/>
       <c r="P27" s="30" t="inlineStr"/>
       <c r="Q27" s="30" t="inlineStr"/>
       <c r="R27" s="30" t="inlineStr"/>
       <c r="S27" s="30" t="inlineStr"/>
-      <c r="T27" s="30" t="inlineStr"/>
+      <c r="T27" s="30" t="inlineStr">
+        <is>
+          <t>24/04/1955</t>
+        </is>
+      </c>
       <c r="U27" s="30" t="inlineStr"/>
       <c r="V27" s="30" t="inlineStr"/>
       <c r="W27" s="30" t="inlineStr"/>
-      <c r="X27" s="30" t="inlineStr"/>
+      <c r="X27" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y27" s="30" t="inlineStr"/>
       <c r="Z27" s="30" t="inlineStr"/>
-      <c r="AA27" s="30" t="inlineStr"/>
+      <c r="AA27" s="30" t="inlineStr">
+        <is>
+          <t>10/04/2024</t>
+        </is>
+      </c>
       <c r="AB27" s="30" t="inlineStr"/>
       <c r="AC27" s="30" t="inlineStr"/>
       <c r="AD27" s="30" t="inlineStr"/>
@@ -4012,7 +4712,11 @@
           <t>9990000027</t>
         </is>
       </c>
-      <c r="E28" s="30" t="inlineStr"/>
+      <c r="E28" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F28" s="30" t="inlineStr"/>
       <c r="G28" s="30" t="inlineStr">
         <is>
@@ -4029,20 +4733,44 @@
       </c>
       <c r="L28" s="30" t="inlineStr"/>
       <c r="M28" s="30" t="inlineStr"/>
-      <c r="N28" s="30" t="inlineStr"/>
+      <c r="N28" s="30" t="inlineStr">
+        <is>
+          <t>27/03/2024</t>
+        </is>
+      </c>
       <c r="O28" s="30" t="inlineStr"/>
       <c r="P28" s="30" t="inlineStr"/>
       <c r="Q28" s="30" t="inlineStr"/>
       <c r="R28" s="30" t="inlineStr"/>
       <c r="S28" s="30" t="inlineStr"/>
-      <c r="T28" s="30" t="inlineStr"/>
-      <c r="U28" s="30" t="inlineStr"/>
-      <c r="V28" s="30" t="inlineStr"/>
+      <c r="T28" s="30" t="inlineStr">
+        <is>
+          <t>22/11/1957</t>
+        </is>
+      </c>
+      <c r="U28" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V28" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W28" s="30" t="inlineStr"/>
-      <c r="X28" s="30" t="inlineStr"/>
+      <c r="X28" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y28" s="30" t="inlineStr"/>
       <c r="Z28" s="30" t="inlineStr"/>
-      <c r="AA28" s="30" t="inlineStr"/>
+      <c r="AA28" s="30" t="inlineStr">
+        <is>
+          <t>22/03/2024</t>
+        </is>
+      </c>
       <c r="AB28" s="30" t="inlineStr"/>
       <c r="AC28" s="30" t="inlineStr"/>
       <c r="AD28" s="30" t="inlineStr"/>
@@ -4118,7 +4846,11 @@
           <t>9990000028</t>
         </is>
       </c>
-      <c r="E29" s="30" t="inlineStr"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="inlineStr"/>
       <c r="G29" s="30" t="inlineStr">
         <is>
@@ -4135,20 +4867,44 @@
       </c>
       <c r="L29" s="30" t="inlineStr"/>
       <c r="M29" s="30" t="inlineStr"/>
-      <c r="N29" s="30" t="inlineStr"/>
+      <c r="N29" s="30" t="inlineStr">
+        <is>
+          <t>16/02/2024</t>
+        </is>
+      </c>
       <c r="O29" s="30" t="inlineStr"/>
       <c r="P29" s="30" t="inlineStr"/>
       <c r="Q29" s="30" t="inlineStr"/>
       <c r="R29" s="30" t="inlineStr"/>
       <c r="S29" s="30" t="inlineStr"/>
-      <c r="T29" s="30" t="inlineStr"/>
-      <c r="U29" s="30" t="inlineStr"/>
-      <c r="V29" s="30" t="inlineStr"/>
+      <c r="T29" s="30" t="inlineStr">
+        <is>
+          <t>22/06/1950</t>
+        </is>
+      </c>
+      <c r="U29" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V29" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W29" s="30" t="inlineStr"/>
-      <c r="X29" s="30" t="inlineStr"/>
+      <c r="X29" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y29" s="30" t="inlineStr"/>
       <c r="Z29" s="30" t="inlineStr"/>
-      <c r="AA29" s="30" t="inlineStr"/>
+      <c r="AA29" s="30" t="inlineStr">
+        <is>
+          <t>04/01/2025</t>
+        </is>
+      </c>
       <c r="AB29" s="30" t="inlineStr"/>
       <c r="AC29" s="30" t="inlineStr"/>
       <c r="AD29" s="30" t="inlineStr"/>
@@ -4167,7 +4923,11 @@
       <c r="AQ29" s="30" t="inlineStr"/>
       <c r="AR29" s="30" t="inlineStr"/>
       <c r="AS29" s="30" t="inlineStr"/>
-      <c r="AT29" s="30" t="inlineStr"/>
+      <c r="AT29" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
       <c r="AU29" s="30" t="inlineStr"/>
       <c r="AV29" s="30" t="inlineStr"/>
       <c r="AW29" s="30" t="inlineStr"/>
@@ -4224,7 +4984,11 @@
           <t>9990000029</t>
         </is>
       </c>
-      <c r="E30" s="30" t="inlineStr"/>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F30" s="30" t="inlineStr"/>
       <c r="G30" s="30" t="inlineStr">
         <is>
@@ -4241,20 +5005,48 @@
       </c>
       <c r="L30" s="30" t="inlineStr"/>
       <c r="M30" s="30" t="inlineStr"/>
-      <c r="N30" s="30" t="inlineStr"/>
+      <c r="N30" s="30" t="inlineStr">
+        <is>
+          <t>07/12/2024</t>
+        </is>
+      </c>
       <c r="O30" s="30" t="inlineStr"/>
       <c r="P30" s="30" t="inlineStr"/>
-      <c r="Q30" s="30" t="inlineStr"/>
+      <c r="Q30" s="30" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
       <c r="R30" s="30" t="inlineStr"/>
       <c r="S30" s="30" t="inlineStr"/>
-      <c r="T30" s="30" t="inlineStr"/>
-      <c r="U30" s="30" t="inlineStr"/>
-      <c r="V30" s="30" t="inlineStr"/>
+      <c r="T30" s="30" t="inlineStr">
+        <is>
+          <t>14/09/1953</t>
+        </is>
+      </c>
+      <c r="U30" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V30" s="30" t="inlineStr">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
       <c r="W30" s="30" t="inlineStr"/>
-      <c r="X30" s="30" t="inlineStr"/>
+      <c r="X30" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y30" s="30" t="inlineStr"/>
       <c r="Z30" s="30" t="inlineStr"/>
-      <c r="AA30" s="30" t="inlineStr"/>
+      <c r="AA30" s="30" t="inlineStr">
+        <is>
+          <t>29/04/2024</t>
+        </is>
+      </c>
       <c r="AB30" s="30" t="inlineStr"/>
       <c r="AC30" s="30" t="inlineStr"/>
       <c r="AD30" s="30" t="inlineStr"/>
@@ -4273,7 +5065,11 @@
       <c r="AQ30" s="30" t="inlineStr"/>
       <c r="AR30" s="30" t="inlineStr"/>
       <c r="AS30" s="30" t="inlineStr"/>
-      <c r="AT30" s="30" t="inlineStr"/>
+      <c r="AT30" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
       <c r="AU30" s="30" t="inlineStr"/>
       <c r="AV30" s="30" t="inlineStr"/>
       <c r="AW30" s="30" t="inlineStr"/>
@@ -4330,7 +5126,11 @@
           <t>9990000030</t>
         </is>
       </c>
-      <c r="E31" s="30" t="inlineStr"/>
+      <c r="E31" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F31" s="30" t="inlineStr"/>
       <c r="G31" s="30" t="inlineStr"/>
       <c r="H31" s="30" t="inlineStr"/>
@@ -4343,20 +5143,48 @@
       </c>
       <c r="L31" s="30" t="inlineStr"/>
       <c r="M31" s="30" t="inlineStr"/>
-      <c r="N31" s="30" t="inlineStr"/>
+      <c r="N31" s="30" t="inlineStr">
+        <is>
+          <t>30/06/2024</t>
+        </is>
+      </c>
       <c r="O31" s="30" t="inlineStr"/>
       <c r="P31" s="30" t="inlineStr"/>
       <c r="Q31" s="30" t="inlineStr"/>
-      <c r="R31" s="30" t="inlineStr"/>
+      <c r="R31" s="30" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
       <c r="S31" s="30" t="inlineStr"/>
-      <c r="T31" s="30" t="inlineStr"/>
-      <c r="U31" s="30" t="inlineStr"/>
-      <c r="V31" s="30" t="inlineStr"/>
+      <c r="T31" s="30" t="inlineStr">
+        <is>
+          <t>12/05/1957</t>
+        </is>
+      </c>
+      <c r="U31" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V31" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W31" s="30" t="inlineStr"/>
-      <c r="X31" s="30" t="inlineStr"/>
+      <c r="X31" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y31" s="30" t="inlineStr"/>
       <c r="Z31" s="30" t="inlineStr"/>
-      <c r="AA31" s="30" t="inlineStr"/>
+      <c r="AA31" s="30" t="inlineStr">
+        <is>
+          <t>13/12/2024</t>
+        </is>
+      </c>
       <c r="AB31" s="30" t="inlineStr"/>
       <c r="AC31" s="30" t="inlineStr"/>
       <c r="AD31" s="30" t="inlineStr"/>
@@ -4376,7 +5204,11 @@
       <c r="AR31" s="30" t="inlineStr"/>
       <c r="AS31" s="30" t="inlineStr"/>
       <c r="AT31" s="30" t="inlineStr"/>
-      <c r="AU31" s="30" t="inlineStr"/>
+      <c r="AU31" s="30" t="inlineStr">
+        <is>
+          <t>15/04/2024</t>
+        </is>
+      </c>
       <c r="AV31" s="30" t="inlineStr"/>
       <c r="AW31" s="30" t="inlineStr"/>
       <c r="AX31" s="30" t="inlineStr"/>
@@ -4432,7 +5264,11 @@
           <t>9990000031</t>
         </is>
       </c>
-      <c r="E32" s="30" t="inlineStr"/>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F32" s="30" t="inlineStr"/>
       <c r="G32" s="30" t="inlineStr">
         <is>
@@ -4440,16 +5276,8 @@
         </is>
       </c>
       <c r="H32" s="30" t="inlineStr"/>
-      <c r="I32" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J32" s="30" t="inlineStr">
-        <is>
-          <t>early annular cancer with abnormal pit pattern opposite ICV</t>
-        </is>
-      </c>
+      <c r="I32" s="30" t="inlineStr"/>
+      <c r="J32" s="30" t="inlineStr"/>
       <c r="K32" s="30" t="inlineStr">
         <is>
           <t>Right‑sided colonic tumour ICD10 Code: D12.6 Differentiation: Moderately differentiated</t>
@@ -4457,20 +5285,44 @@
       </c>
       <c r="L32" s="30" t="inlineStr"/>
       <c r="M32" s="30" t="inlineStr"/>
-      <c r="N32" s="30" t="inlineStr"/>
+      <c r="N32" s="30" t="inlineStr">
+        <is>
+          <t>13/02/2025</t>
+        </is>
+      </c>
       <c r="O32" s="30" t="inlineStr"/>
       <c r="P32" s="30" t="inlineStr"/>
       <c r="Q32" s="30" t="inlineStr"/>
       <c r="R32" s="30" t="inlineStr"/>
       <c r="S32" s="30" t="inlineStr"/>
-      <c r="T32" s="30" t="inlineStr"/>
-      <c r="U32" s="30" t="inlineStr"/>
-      <c r="V32" s="30" t="inlineStr"/>
+      <c r="T32" s="30" t="inlineStr">
+        <is>
+          <t>18/11/1953</t>
+        </is>
+      </c>
+      <c r="U32" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V32" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W32" s="30" t="inlineStr"/>
-      <c r="X32" s="30" t="inlineStr"/>
+      <c r="X32" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y32" s="30" t="inlineStr"/>
       <c r="Z32" s="30" t="inlineStr"/>
-      <c r="AA32" s="30" t="inlineStr"/>
+      <c r="AA32" s="30" t="inlineStr">
+        <is>
+          <t>13/05/2024</t>
+        </is>
+      </c>
       <c r="AB32" s="30" t="inlineStr"/>
       <c r="AC32" s="30" t="inlineStr"/>
       <c r="AD32" s="30" t="inlineStr"/>
@@ -4489,8 +5341,16 @@
       <c r="AQ32" s="30" t="inlineStr"/>
       <c r="AR32" s="30" t="inlineStr"/>
       <c r="AS32" s="30" t="inlineStr"/>
-      <c r="AT32" s="30" t="inlineStr"/>
-      <c r="AU32" s="30" t="inlineStr"/>
+      <c r="AT32" s="30" t="inlineStr">
+        <is>
+          <t>hemicolectomy</t>
+        </is>
+      </c>
+      <c r="AU32" s="30" t="inlineStr">
+        <is>
+          <t>06/12/2024</t>
+        </is>
+      </c>
       <c r="AV32" s="30" t="inlineStr"/>
       <c r="AW32" s="30" t="inlineStr"/>
       <c r="AX32" s="30" t="inlineStr"/>
@@ -4546,7 +5406,11 @@
           <t>9990000032</t>
         </is>
       </c>
-      <c r="E33" s="30" t="inlineStr"/>
+      <c r="E33" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F33" s="30" t="inlineStr"/>
       <c r="G33" s="30" t="inlineStr"/>
       <c r="H33" s="30" t="inlineStr"/>
@@ -4559,20 +5423,44 @@
       </c>
       <c r="L33" s="30" t="inlineStr"/>
       <c r="M33" s="30" t="inlineStr"/>
-      <c r="N33" s="30" t="inlineStr"/>
+      <c r="N33" s="30" t="inlineStr">
+        <is>
+          <t>29/04/2024</t>
+        </is>
+      </c>
       <c r="O33" s="30" t="inlineStr"/>
       <c r="P33" s="30" t="inlineStr"/>
       <c r="Q33" s="30" t="inlineStr"/>
       <c r="R33" s="30" t="inlineStr"/>
       <c r="S33" s="30" t="inlineStr"/>
-      <c r="T33" s="30" t="inlineStr"/>
-      <c r="U33" s="30" t="inlineStr"/>
-      <c r="V33" s="30" t="inlineStr"/>
+      <c r="T33" s="30" t="inlineStr">
+        <is>
+          <t>14/02/1967</t>
+        </is>
+      </c>
+      <c r="U33" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V33" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W33" s="30" t="inlineStr"/>
-      <c r="X33" s="30" t="inlineStr"/>
+      <c r="X33" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y33" s="30" t="inlineStr"/>
       <c r="Z33" s="30" t="inlineStr"/>
-      <c r="AA33" s="30" t="inlineStr"/>
+      <c r="AA33" s="30" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
       <c r="AB33" s="30" t="inlineStr"/>
       <c r="AC33" s="30" t="inlineStr"/>
       <c r="AD33" s="30" t="inlineStr"/>
@@ -4591,7 +5479,11 @@
       <c r="AQ33" s="30" t="inlineStr"/>
       <c r="AR33" s="30" t="inlineStr"/>
       <c r="AS33" s="30" t="inlineStr"/>
-      <c r="AT33" s="30" t="inlineStr"/>
+      <c r="AT33" s="30" t="inlineStr">
+        <is>
+          <t>surgery</t>
+        </is>
+      </c>
       <c r="AU33" s="30" t="inlineStr"/>
       <c r="AV33" s="30" t="inlineStr"/>
       <c r="AW33" s="30" t="inlineStr"/>
@@ -4648,7 +5540,11 @@
           <t>9990000033</t>
         </is>
       </c>
-      <c r="E34" s="30" t="inlineStr"/>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F34" s="30" t="inlineStr"/>
       <c r="G34" s="30" t="inlineStr"/>
       <c r="H34" s="30" t="inlineStr"/>
@@ -4661,20 +5557,44 @@
       </c>
       <c r="L34" s="30" t="inlineStr"/>
       <c r="M34" s="30" t="inlineStr"/>
-      <c r="N34" s="30" t="inlineStr"/>
+      <c r="N34" s="30" t="inlineStr">
+        <is>
+          <t>25/03/2024</t>
+        </is>
+      </c>
       <c r="O34" s="30" t="inlineStr"/>
       <c r="P34" s="30" t="inlineStr"/>
       <c r="Q34" s="30" t="inlineStr"/>
       <c r="R34" s="30" t="inlineStr"/>
       <c r="S34" s="30" t="inlineStr"/>
-      <c r="T34" s="30" t="inlineStr"/>
-      <c r="U34" s="30" t="inlineStr"/>
-      <c r="V34" s="30" t="inlineStr"/>
+      <c r="T34" s="30" t="inlineStr">
+        <is>
+          <t>15/11/1967</t>
+        </is>
+      </c>
+      <c r="U34" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V34" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W34" s="30" t="inlineStr"/>
-      <c r="X34" s="30" t="inlineStr"/>
+      <c r="X34" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y34" s="30" t="inlineStr"/>
       <c r="Z34" s="30" t="inlineStr"/>
-      <c r="AA34" s="30" t="inlineStr"/>
+      <c r="AA34" s="30" t="inlineStr">
+        <is>
+          <t>05/03/2024</t>
+        </is>
+      </c>
       <c r="AB34" s="30" t="inlineStr"/>
       <c r="AC34" s="30" t="inlineStr"/>
       <c r="AD34" s="30" t="inlineStr"/>
@@ -4693,7 +5613,11 @@
       <c r="AQ34" s="30" t="inlineStr"/>
       <c r="AR34" s="30" t="inlineStr"/>
       <c r="AS34" s="30" t="inlineStr"/>
-      <c r="AT34" s="30" t="inlineStr"/>
+      <c r="AT34" s="30" t="inlineStr">
+        <is>
+          <t>hemicolectomy</t>
+        </is>
+      </c>
       <c r="AU34" s="30" t="inlineStr"/>
       <c r="AV34" s="30" t="inlineStr"/>
       <c r="AW34" s="30" t="inlineStr"/>
@@ -4750,7 +5674,11 @@
           <t>9990000034</t>
         </is>
       </c>
-      <c r="E35" s="30" t="inlineStr"/>
+      <c r="E35" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F35" s="30" t="inlineStr"/>
       <c r="G35" s="30" t="inlineStr"/>
       <c r="H35" s="30" t="inlineStr"/>
@@ -4763,20 +5691,44 @@
       </c>
       <c r="L35" s="30" t="inlineStr"/>
       <c r="M35" s="30" t="inlineStr"/>
-      <c r="N35" s="30" t="inlineStr"/>
+      <c r="N35" s="30" t="inlineStr">
+        <is>
+          <t>06/05/2024</t>
+        </is>
+      </c>
       <c r="O35" s="30" t="inlineStr"/>
       <c r="P35" s="30" t="inlineStr"/>
       <c r="Q35" s="30" t="inlineStr"/>
       <c r="R35" s="30" t="inlineStr"/>
       <c r="S35" s="30" t="inlineStr"/>
-      <c r="T35" s="30" t="inlineStr"/>
-      <c r="U35" s="30" t="inlineStr"/>
-      <c r="V35" s="30" t="inlineStr"/>
+      <c r="T35" s="30" t="inlineStr">
+        <is>
+          <t>22/07/1976</t>
+        </is>
+      </c>
+      <c r="U35" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V35" s="30" t="inlineStr">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
       <c r="W35" s="30" t="inlineStr"/>
-      <c r="X35" s="30" t="inlineStr"/>
+      <c r="X35" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y35" s="30" t="inlineStr"/>
       <c r="Z35" s="30" t="inlineStr"/>
-      <c r="AA35" s="30" t="inlineStr"/>
+      <c r="AA35" s="30" t="inlineStr">
+        <is>
+          <t>23/04/2024</t>
+        </is>
+      </c>
       <c r="AB35" s="30" t="inlineStr"/>
       <c r="AC35" s="30" t="inlineStr"/>
       <c r="AD35" s="30" t="inlineStr"/>
@@ -4796,7 +5748,11 @@
       <c r="AR35" s="30" t="inlineStr"/>
       <c r="AS35" s="30" t="inlineStr"/>
       <c r="AT35" s="30" t="inlineStr"/>
-      <c r="AU35" s="30" t="inlineStr"/>
+      <c r="AU35" s="30" t="inlineStr">
+        <is>
+          <t>13/02/2024</t>
+        </is>
+      </c>
       <c r="AV35" s="30" t="inlineStr"/>
       <c r="AW35" s="30" t="inlineStr"/>
       <c r="AX35" s="30" t="inlineStr"/>
@@ -4852,7 +5808,11 @@
           <t>9990000035</t>
         </is>
       </c>
-      <c r="E36" s="30" t="inlineStr"/>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F36" s="30" t="inlineStr"/>
       <c r="G36" s="30" t="inlineStr"/>
       <c r="H36" s="30" t="inlineStr"/>
@@ -4865,20 +5825,44 @@
       </c>
       <c r="L36" s="30" t="inlineStr"/>
       <c r="M36" s="30" t="inlineStr"/>
-      <c r="N36" s="30" t="inlineStr"/>
+      <c r="N36" s="30" t="inlineStr">
+        <is>
+          <t>24/06/2024</t>
+        </is>
+      </c>
       <c r="O36" s="30" t="inlineStr"/>
       <c r="P36" s="30" t="inlineStr"/>
       <c r="Q36" s="30" t="inlineStr"/>
       <c r="R36" s="30" t="inlineStr"/>
       <c r="S36" s="30" t="inlineStr"/>
-      <c r="T36" s="30" t="inlineStr"/>
-      <c r="U36" s="30" t="inlineStr"/>
-      <c r="V36" s="30" t="inlineStr"/>
+      <c r="T36" s="30" t="inlineStr">
+        <is>
+          <t>20/12/1967</t>
+        </is>
+      </c>
+      <c r="U36" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V36" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W36" s="30" t="inlineStr"/>
-      <c r="X36" s="30" t="inlineStr"/>
+      <c r="X36" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y36" s="30" t="inlineStr"/>
       <c r="Z36" s="30" t="inlineStr"/>
-      <c r="AA36" s="30" t="inlineStr"/>
+      <c r="AA36" s="30" t="inlineStr">
+        <is>
+          <t>21/01/2024</t>
+        </is>
+      </c>
       <c r="AB36" s="30" t="inlineStr"/>
       <c r="AC36" s="30" t="inlineStr"/>
       <c r="AD36" s="30" t="inlineStr"/>
@@ -4898,7 +5882,11 @@
       <c r="AR36" s="30" t="inlineStr"/>
       <c r="AS36" s="30" t="inlineStr"/>
       <c r="AT36" s="30" t="inlineStr"/>
-      <c r="AU36" s="30" t="inlineStr"/>
+      <c r="AU36" s="30" t="inlineStr">
+        <is>
+          <t>09/04/2024</t>
+        </is>
+      </c>
       <c r="AV36" s="30" t="inlineStr"/>
       <c r="AW36" s="30" t="inlineStr"/>
       <c r="AX36" s="30" t="inlineStr"/>
@@ -4954,7 +5942,11 @@
           <t>9990000036</t>
         </is>
       </c>
-      <c r="E37" s="30" t="inlineStr"/>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F37" s="30" t="inlineStr"/>
       <c r="G37" s="30" t="inlineStr"/>
       <c r="H37" s="30" t="inlineStr"/>
@@ -4967,20 +5959,44 @@
       </c>
       <c r="L37" s="30" t="inlineStr"/>
       <c r="M37" s="30" t="inlineStr"/>
-      <c r="N37" s="30" t="inlineStr"/>
+      <c r="N37" s="30" t="inlineStr">
+        <is>
+          <t>01/01/2024</t>
+        </is>
+      </c>
       <c r="O37" s="30" t="inlineStr"/>
       <c r="P37" s="30" t="inlineStr"/>
       <c r="Q37" s="30" t="inlineStr"/>
       <c r="R37" s="30" t="inlineStr"/>
       <c r="S37" s="30" t="inlineStr"/>
-      <c r="T37" s="30" t="inlineStr"/>
-      <c r="U37" s="30" t="inlineStr"/>
-      <c r="V37" s="30" t="inlineStr"/>
+      <c r="T37" s="30" t="inlineStr">
+        <is>
+          <t>04/07/1981</t>
+        </is>
+      </c>
+      <c r="U37" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V37" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W37" s="30" t="inlineStr"/>
-      <c r="X37" s="30" t="inlineStr"/>
+      <c r="X37" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y37" s="30" t="inlineStr"/>
       <c r="Z37" s="30" t="inlineStr"/>
-      <c r="AA37" s="30" t="inlineStr"/>
+      <c r="AA37" s="30" t="inlineStr">
+        <is>
+          <t>14/06/2024</t>
+        </is>
+      </c>
       <c r="AB37" s="30" t="inlineStr"/>
       <c r="AC37" s="30" t="inlineStr"/>
       <c r="AD37" s="30" t="inlineStr"/>
@@ -4999,8 +6015,16 @@
       <c r="AQ37" s="30" t="inlineStr"/>
       <c r="AR37" s="30" t="inlineStr"/>
       <c r="AS37" s="30" t="inlineStr"/>
-      <c r="AT37" s="30" t="inlineStr"/>
-      <c r="AU37" s="30" t="inlineStr"/>
+      <c r="AT37" s="30" t="inlineStr">
+        <is>
+          <t>hemicolectomy</t>
+        </is>
+      </c>
+      <c r="AU37" s="30" t="inlineStr">
+        <is>
+          <t>07/01/2024</t>
+        </is>
+      </c>
       <c r="AV37" s="30" t="inlineStr"/>
       <c r="AW37" s="30" t="inlineStr"/>
       <c r="AX37" s="30" t="inlineStr"/>
@@ -5056,7 +6080,11 @@
           <t>9990000037</t>
         </is>
       </c>
-      <c r="E38" s="30" t="inlineStr"/>
+      <c r="E38" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F38" s="30" t="inlineStr"/>
       <c r="G38" s="30" t="inlineStr">
         <is>
@@ -5064,16 +6092,8 @@
         </is>
       </c>
       <c r="H38" s="30" t="inlineStr"/>
-      <c r="I38" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J38" s="30" t="inlineStr">
-        <is>
-          <t>multiple polyps, is there a history of a polyposis syndrome? Suspicious cancers in the transverse and ascending colons.</t>
-        </is>
-      </c>
+      <c r="I38" s="30" t="inlineStr"/>
+      <c r="J38" s="30" t="inlineStr"/>
       <c r="K38" s="30" t="inlineStr">
         <is>
           <t>Right‑sided colonic tumour ICD10 Code: C18.0 Differentiation: Poorly differentiated</t>
@@ -5081,20 +6101,44 @@
       </c>
       <c r="L38" s="30" t="inlineStr"/>
       <c r="M38" s="30" t="inlineStr"/>
-      <c r="N38" s="30" t="inlineStr"/>
+      <c r="N38" s="30" t="inlineStr">
+        <is>
+          <t>15/08/2024</t>
+        </is>
+      </c>
       <c r="O38" s="30" t="inlineStr"/>
       <c r="P38" s="30" t="inlineStr"/>
       <c r="Q38" s="30" t="inlineStr"/>
       <c r="R38" s="30" t="inlineStr"/>
       <c r="S38" s="30" t="inlineStr"/>
-      <c r="T38" s="30" t="inlineStr"/>
-      <c r="U38" s="30" t="inlineStr"/>
-      <c r="V38" s="30" t="inlineStr"/>
+      <c r="T38" s="30" t="inlineStr">
+        <is>
+          <t>06/10/1947</t>
+        </is>
+      </c>
+      <c r="U38" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V38" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W38" s="30" t="inlineStr"/>
-      <c r="X38" s="30" t="inlineStr"/>
+      <c r="X38" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y38" s="30" t="inlineStr"/>
       <c r="Z38" s="30" t="inlineStr"/>
-      <c r="AA38" s="30" t="inlineStr"/>
+      <c r="AA38" s="30" t="inlineStr">
+        <is>
+          <t>24/09/2024</t>
+        </is>
+      </c>
       <c r="AB38" s="30" t="inlineStr"/>
       <c r="AC38" s="30" t="inlineStr"/>
       <c r="AD38" s="30" t="inlineStr"/>
@@ -5170,20 +6214,16 @@
           <t>9990000038</t>
         </is>
       </c>
-      <c r="E39" s="30" t="inlineStr"/>
+      <c r="E39" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F39" s="30" t="inlineStr"/>
       <c r="G39" s="30" t="inlineStr"/>
       <c r="H39" s="30" t="inlineStr"/>
-      <c r="I39" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J39" s="30" t="inlineStr">
-        <is>
-          <t>sessile lesion in re</t>
-        </is>
-      </c>
+      <c r="I39" s="30" t="inlineStr"/>
+      <c r="J39" s="30" t="inlineStr"/>
       <c r="K39" s="30" t="inlineStr">
         <is>
           <t>Villous adenoma with focal invasion ICD10 Code: C19 Differentiation: Poorly differentiated</t>
@@ -5191,20 +6231,44 @@
       </c>
       <c r="L39" s="30" t="inlineStr"/>
       <c r="M39" s="30" t="inlineStr"/>
-      <c r="N39" s="30" t="inlineStr"/>
+      <c r="N39" s="30" t="inlineStr">
+        <is>
+          <t>25/11/2024</t>
+        </is>
+      </c>
       <c r="O39" s="30" t="inlineStr"/>
       <c r="P39" s="30" t="inlineStr"/>
       <c r="Q39" s="30" t="inlineStr"/>
       <c r="R39" s="30" t="inlineStr"/>
       <c r="S39" s="30" t="inlineStr"/>
-      <c r="T39" s="30" t="inlineStr"/>
-      <c r="U39" s="30" t="inlineStr"/>
-      <c r="V39" s="30" t="inlineStr"/>
+      <c r="T39" s="30" t="inlineStr">
+        <is>
+          <t>07/09/1975</t>
+        </is>
+      </c>
+      <c r="U39" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V39" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W39" s="30" t="inlineStr"/>
-      <c r="X39" s="30" t="inlineStr"/>
+      <c r="X39" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y39" s="30" t="inlineStr"/>
       <c r="Z39" s="30" t="inlineStr"/>
-      <c r="AA39" s="30" t="inlineStr"/>
+      <c r="AA39" s="30" t="inlineStr">
+        <is>
+          <t>17/03/2024</t>
+        </is>
+      </c>
       <c r="AB39" s="30" t="inlineStr"/>
       <c r="AC39" s="30" t="inlineStr"/>
       <c r="AD39" s="30" t="inlineStr"/>
@@ -5280,7 +6344,11 @@
           <t>9990000039</t>
         </is>
       </c>
-      <c r="E40" s="30" t="inlineStr"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F40" s="30" t="inlineStr"/>
       <c r="G40" s="30" t="inlineStr">
         <is>
@@ -5297,20 +6365,44 @@
       </c>
       <c r="L40" s="30" t="inlineStr"/>
       <c r="M40" s="30" t="inlineStr"/>
-      <c r="N40" s="30" t="inlineStr"/>
+      <c r="N40" s="30" t="inlineStr">
+        <is>
+          <t>18/02/2024</t>
+        </is>
+      </c>
       <c r="O40" s="30" t="inlineStr"/>
       <c r="P40" s="30" t="inlineStr"/>
       <c r="Q40" s="30" t="inlineStr"/>
       <c r="R40" s="30" t="inlineStr"/>
       <c r="S40" s="30" t="inlineStr"/>
-      <c r="T40" s="30" t="inlineStr"/>
-      <c r="U40" s="30" t="inlineStr"/>
-      <c r="V40" s="30" t="inlineStr"/>
+      <c r="T40" s="30" t="inlineStr">
+        <is>
+          <t>05/03/1949</t>
+        </is>
+      </c>
+      <c r="U40" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V40" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W40" s="30" t="inlineStr"/>
-      <c r="X40" s="30" t="inlineStr"/>
+      <c r="X40" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y40" s="30" t="inlineStr"/>
       <c r="Z40" s="30" t="inlineStr"/>
-      <c r="AA40" s="30" t="inlineStr"/>
+      <c r="AA40" s="30" t="inlineStr">
+        <is>
+          <t>14/10/2024</t>
+        </is>
+      </c>
       <c r="AB40" s="30" t="inlineStr"/>
       <c r="AC40" s="30" t="inlineStr"/>
       <c r="AD40" s="30" t="inlineStr"/>
@@ -5329,7 +6421,11 @@
       <c r="AQ40" s="30" t="inlineStr"/>
       <c r="AR40" s="30" t="inlineStr"/>
       <c r="AS40" s="30" t="inlineStr"/>
-      <c r="AT40" s="30" t="inlineStr"/>
+      <c r="AT40" s="30" t="inlineStr">
+        <is>
+          <t>hemicolectomy</t>
+        </is>
+      </c>
       <c r="AU40" s="30" t="inlineStr"/>
       <c r="AV40" s="30" t="inlineStr"/>
       <c r="AW40" s="30" t="inlineStr"/>
@@ -5386,20 +6482,16 @@
           <t>9990000040</t>
         </is>
       </c>
-      <c r="E41" s="30" t="inlineStr"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F41" s="30" t="inlineStr"/>
       <c r="G41" s="30" t="inlineStr"/>
       <c r="H41" s="30" t="inlineStr"/>
-      <c r="I41" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J41" s="30" t="inlineStr">
-        <is>
-          <t>polypoidal lesion in cecum</t>
-        </is>
-      </c>
+      <c r="I41" s="30" t="inlineStr"/>
+      <c r="J41" s="30" t="inlineStr"/>
       <c r="K41" s="30" t="inlineStr">
         <is>
           <t>Caecal adenocarcinoma ICD10 Code: C18.2 Differentiation: Moderately differentiated</t>
@@ -5407,20 +6499,40 @@
       </c>
       <c r="L41" s="30" t="inlineStr"/>
       <c r="M41" s="30" t="inlineStr"/>
-      <c r="N41" s="30" t="inlineStr"/>
+      <c r="N41" s="30" t="inlineStr">
+        <is>
+          <t>15/12/2024</t>
+        </is>
+      </c>
       <c r="O41" s="30" t="inlineStr"/>
       <c r="P41" s="30" t="inlineStr"/>
       <c r="Q41" s="30" t="inlineStr"/>
       <c r="R41" s="30" t="inlineStr"/>
       <c r="S41" s="30" t="inlineStr"/>
-      <c r="T41" s="30" t="inlineStr"/>
+      <c r="T41" s="30" t="inlineStr">
+        <is>
+          <t>08/08/1956</t>
+        </is>
+      </c>
       <c r="U41" s="30" t="inlineStr"/>
-      <c r="V41" s="30" t="inlineStr"/>
+      <c r="V41" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W41" s="30" t="inlineStr"/>
-      <c r="X41" s="30" t="inlineStr"/>
+      <c r="X41" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y41" s="30" t="inlineStr"/>
       <c r="Z41" s="30" t="inlineStr"/>
-      <c r="AA41" s="30" t="inlineStr"/>
+      <c r="AA41" s="30" t="inlineStr">
+        <is>
+          <t>17/11/2024</t>
+        </is>
+      </c>
       <c r="AB41" s="30" t="inlineStr"/>
       <c r="AC41" s="30" t="inlineStr"/>
       <c r="AD41" s="30" t="inlineStr"/>
@@ -5496,7 +6608,11 @@
           <t>9990000041</t>
         </is>
       </c>
-      <c r="E42" s="30" t="inlineStr"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F42" s="30" t="inlineStr"/>
       <c r="G42" s="30" t="inlineStr"/>
       <c r="H42" s="30" t="inlineStr"/>
@@ -5509,20 +6625,44 @@
       </c>
       <c r="L42" s="30" t="inlineStr"/>
       <c r="M42" s="30" t="inlineStr"/>
-      <c r="N42" s="30" t="inlineStr"/>
+      <c r="N42" s="30" t="inlineStr">
+        <is>
+          <t>18/01/2025</t>
+        </is>
+      </c>
       <c r="O42" s="30" t="inlineStr"/>
       <c r="P42" s="30" t="inlineStr"/>
       <c r="Q42" s="30" t="inlineStr"/>
       <c r="R42" s="30" t="inlineStr"/>
       <c r="S42" s="30" t="inlineStr"/>
-      <c r="T42" s="30" t="inlineStr"/>
-      <c r="U42" s="30" t="inlineStr"/>
-      <c r="V42" s="30" t="inlineStr"/>
+      <c r="T42" s="30" t="inlineStr">
+        <is>
+          <t>09/10/1970</t>
+        </is>
+      </c>
+      <c r="U42" s="30" t="inlineStr">
+        <is>
+          <t>3c</t>
+        </is>
+      </c>
+      <c r="V42" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W42" s="30" t="inlineStr"/>
-      <c r="X42" s="30" t="inlineStr"/>
+      <c r="X42" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y42" s="30" t="inlineStr"/>
       <c r="Z42" s="30" t="inlineStr"/>
-      <c r="AA42" s="30" t="inlineStr"/>
+      <c r="AA42" s="30" t="inlineStr">
+        <is>
+          <t>07/04/2024</t>
+        </is>
+      </c>
       <c r="AB42" s="30" t="inlineStr"/>
       <c r="AC42" s="30" t="inlineStr"/>
       <c r="AD42" s="30" t="inlineStr"/>
@@ -5542,7 +6682,11 @@
       <c r="AR42" s="30" t="inlineStr"/>
       <c r="AS42" s="30" t="inlineStr"/>
       <c r="AT42" s="30" t="inlineStr"/>
-      <c r="AU42" s="30" t="inlineStr"/>
+      <c r="AU42" s="30" t="inlineStr">
+        <is>
+          <t>20/10/2024</t>
+        </is>
+      </c>
       <c r="AV42" s="30" t="inlineStr"/>
       <c r="AW42" s="30" t="inlineStr"/>
       <c r="AX42" s="30" t="inlineStr"/>
@@ -5552,7 +6696,11 @@
       <c r="BB42" s="30" t="inlineStr"/>
       <c r="BC42" s="30" t="inlineStr"/>
       <c r="BD42" s="30" t="inlineStr"/>
-      <c r="BE42" s="30" t="inlineStr"/>
+      <c r="BE42" s="30" t="inlineStr">
+        <is>
+          <t>03/11/2024</t>
+        </is>
+      </c>
       <c r="BF42" s="30" t="inlineStr"/>
       <c r="BG42" s="30" t="inlineStr"/>
       <c r="BH42" s="30" t="inlineStr"/>
@@ -5598,20 +6746,16 @@
           <t>9990000042</t>
         </is>
       </c>
-      <c r="E43" s="30" t="inlineStr"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F43" s="30" t="inlineStr"/>
       <c r="G43" s="30" t="inlineStr"/>
       <c r="H43" s="30" t="inlineStr"/>
-      <c r="I43" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J43" s="30" t="inlineStr">
-        <is>
-          <t>polypoidal lesion in sigmoid colon</t>
-        </is>
-      </c>
+      <c r="I43" s="30" t="inlineStr"/>
+      <c r="J43" s="30" t="inlineStr"/>
       <c r="K43" s="30" t="inlineStr">
         <is>
           <t>Large sessile polyp with possible malignant change ICD10 Code: C18.2 Differentiation: Well differentiated</t>
@@ -5625,14 +6769,30 @@
       <c r="Q43" s="30" t="inlineStr"/>
       <c r="R43" s="30" t="inlineStr"/>
       <c r="S43" s="30" t="inlineStr"/>
-      <c r="T43" s="30" t="inlineStr"/>
+      <c r="T43" s="30" t="inlineStr">
+        <is>
+          <t>13/07/1958</t>
+        </is>
+      </c>
       <c r="U43" s="30" t="inlineStr"/>
-      <c r="V43" s="30" t="inlineStr"/>
+      <c r="V43" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W43" s="30" t="inlineStr"/>
-      <c r="X43" s="30" t="inlineStr"/>
+      <c r="X43" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y43" s="30" t="inlineStr"/>
       <c r="Z43" s="30" t="inlineStr"/>
-      <c r="AA43" s="30" t="inlineStr"/>
+      <c r="AA43" s="30" t="inlineStr">
+        <is>
+          <t>01/07/2024</t>
+        </is>
+      </c>
       <c r="AB43" s="30" t="inlineStr"/>
       <c r="AC43" s="30" t="inlineStr"/>
       <c r="AD43" s="30" t="inlineStr"/>
@@ -5651,7 +6811,11 @@
       <c r="AQ43" s="30" t="inlineStr"/>
       <c r="AR43" s="30" t="inlineStr"/>
       <c r="AS43" s="30" t="inlineStr"/>
-      <c r="AT43" s="30" t="inlineStr"/>
+      <c r="AT43" s="30" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
       <c r="AU43" s="30" t="inlineStr"/>
       <c r="AV43" s="30" t="inlineStr"/>
       <c r="AW43" s="30" t="inlineStr"/>
@@ -5708,7 +6872,11 @@
           <t>9990000043</t>
         </is>
       </c>
-      <c r="E44" s="30" t="inlineStr"/>
+      <c r="E44" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F44" s="30" t="inlineStr"/>
       <c r="G44" s="30" t="inlineStr"/>
       <c r="H44" s="30" t="inlineStr"/>
@@ -5721,20 +6889,44 @@
       </c>
       <c r="L44" s="30" t="inlineStr"/>
       <c r="M44" s="30" t="inlineStr"/>
-      <c r="N44" s="30" t="inlineStr"/>
+      <c r="N44" s="30" t="inlineStr">
+        <is>
+          <t>10/06/2024</t>
+        </is>
+      </c>
       <c r="O44" s="30" t="inlineStr"/>
       <c r="P44" s="30" t="inlineStr"/>
       <c r="Q44" s="30" t="inlineStr"/>
       <c r="R44" s="30" t="inlineStr"/>
       <c r="S44" s="30" t="inlineStr"/>
-      <c r="T44" s="30" t="inlineStr"/>
-      <c r="U44" s="30" t="inlineStr"/>
-      <c r="V44" s="30" t="inlineStr"/>
+      <c r="T44" s="30" t="inlineStr">
+        <is>
+          <t>22/06/1962</t>
+        </is>
+      </c>
+      <c r="U44" s="30" t="inlineStr">
+        <is>
+          <t>4a</t>
+        </is>
+      </c>
+      <c r="V44" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W44" s="30" t="inlineStr"/>
-      <c r="X44" s="30" t="inlineStr"/>
+      <c r="X44" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y44" s="30" t="inlineStr"/>
       <c r="Z44" s="30" t="inlineStr"/>
-      <c r="AA44" s="30" t="inlineStr"/>
+      <c r="AA44" s="30" t="inlineStr">
+        <is>
+          <t>17/11/2024</t>
+        </is>
+      </c>
       <c r="AB44" s="30" t="inlineStr"/>
       <c r="AC44" s="30" t="inlineStr"/>
       <c r="AD44" s="30" t="inlineStr"/>
@@ -5802,7 +6994,11 @@
       <c r="B45" s="30" t="inlineStr"/>
       <c r="C45" s="30" t="inlineStr"/>
       <c r="D45" s="30" t="inlineStr"/>
-      <c r="E45" s="30" t="inlineStr"/>
+      <c r="E45" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F45" s="30" t="inlineStr"/>
       <c r="G45" s="30" t="inlineStr"/>
       <c r="H45" s="30" t="inlineStr"/>
@@ -5815,20 +7011,36 @@
       </c>
       <c r="L45" s="30" t="inlineStr"/>
       <c r="M45" s="30" t="inlineStr"/>
-      <c r="N45" s="30" t="inlineStr"/>
+      <c r="N45" s="30" t="inlineStr">
+        <is>
+          <t>18/01/2025</t>
+        </is>
+      </c>
       <c r="O45" s="30" t="inlineStr"/>
       <c r="P45" s="30" t="inlineStr"/>
       <c r="Q45" s="30" t="inlineStr"/>
       <c r="R45" s="30" t="inlineStr"/>
       <c r="S45" s="30" t="inlineStr"/>
-      <c r="T45" s="30" t="inlineStr"/>
+      <c r="T45" s="30" t="inlineStr">
+        <is>
+          <t>06/05/1971</t>
+        </is>
+      </c>
       <c r="U45" s="30" t="inlineStr"/>
       <c r="V45" s="30" t="inlineStr"/>
       <c r="W45" s="30" t="inlineStr"/>
-      <c r="X45" s="30" t="inlineStr"/>
+      <c r="X45" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y45" s="30" t="inlineStr"/>
       <c r="Z45" s="30" t="inlineStr"/>
-      <c r="AA45" s="30" t="inlineStr"/>
+      <c r="AA45" s="30" t="inlineStr">
+        <is>
+          <t>22/06/2024</t>
+        </is>
+      </c>
       <c r="AB45" s="30" t="inlineStr"/>
       <c r="AC45" s="30" t="inlineStr"/>
       <c r="AD45" s="30" t="inlineStr"/>
@@ -5904,7 +7116,11 @@
           <t>9990000045</t>
         </is>
       </c>
-      <c r="E46" s="30" t="inlineStr"/>
+      <c r="E46" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F46" s="30" t="inlineStr"/>
       <c r="G46" s="30" t="inlineStr">
         <is>
@@ -5912,16 +7128,8 @@
         </is>
       </c>
       <c r="H46" s="30" t="inlineStr"/>
-      <c r="I46" s="30" t="inlineStr">
-        <is>
-          <t>Colonoscopy</t>
-        </is>
-      </c>
-      <c r="J46" s="30" t="inlineStr">
-        <is>
-          <t>tumour at 18 cm, biopsied</t>
-        </is>
-      </c>
+      <c r="I46" s="30" t="inlineStr"/>
+      <c r="J46" s="30" t="inlineStr"/>
       <c r="K46" s="30" t="inlineStr">
         <is>
           <t>Right‑sided colonic tumour ICD10 Code: C18.4 Differentiation: Moderately differentiated</t>
@@ -5929,20 +7137,44 @@
       </c>
       <c r="L46" s="30" t="inlineStr"/>
       <c r="M46" s="30" t="inlineStr"/>
-      <c r="N46" s="30" t="inlineStr"/>
+      <c r="N46" s="30" t="inlineStr">
+        <is>
+          <t>23/08/2024</t>
+        </is>
+      </c>
       <c r="O46" s="30" t="inlineStr"/>
       <c r="P46" s="30" t="inlineStr"/>
       <c r="Q46" s="30" t="inlineStr"/>
       <c r="R46" s="30" t="inlineStr"/>
       <c r="S46" s="30" t="inlineStr"/>
-      <c r="T46" s="30" t="inlineStr"/>
-      <c r="U46" s="30" t="inlineStr"/>
-      <c r="V46" s="30" t="inlineStr"/>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>16/11/1982</t>
+        </is>
+      </c>
+      <c r="U46" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V46" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="W46" s="30" t="inlineStr"/>
-      <c r="X46" s="30" t="inlineStr"/>
+      <c r="X46" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y46" s="30" t="inlineStr"/>
       <c r="Z46" s="30" t="inlineStr"/>
-      <c r="AA46" s="30" t="inlineStr"/>
+      <c r="AA46" s="30" t="inlineStr">
+        <is>
+          <t>12/11/2024</t>
+        </is>
+      </c>
       <c r="AB46" s="30" t="inlineStr"/>
       <c r="AC46" s="30" t="inlineStr"/>
       <c r="AD46" s="30" t="inlineStr"/>
@@ -5961,7 +7193,11 @@
       <c r="AQ46" s="30" t="inlineStr"/>
       <c r="AR46" s="30" t="inlineStr"/>
       <c r="AS46" s="30" t="inlineStr"/>
-      <c r="AT46" s="30" t="inlineStr"/>
+      <c r="AT46" s="30" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
       <c r="AU46" s="30" t="inlineStr"/>
       <c r="AV46" s="30" t="inlineStr"/>
       <c r="AW46" s="30" t="inlineStr"/>
@@ -6018,7 +7254,11 @@
           <t>9990000046</t>
         </is>
       </c>
-      <c r="E47" s="30" t="inlineStr"/>
+      <c r="E47" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F47" s="30" t="inlineStr"/>
       <c r="G47" s="30" t="inlineStr"/>
       <c r="H47" s="30" t="inlineStr"/>
@@ -6031,20 +7271,44 @@
       </c>
       <c r="L47" s="30" t="inlineStr"/>
       <c r="M47" s="30" t="inlineStr"/>
-      <c r="N47" s="30" t="inlineStr"/>
+      <c r="N47" s="30" t="inlineStr">
+        <is>
+          <t>13/01/2025</t>
+        </is>
+      </c>
       <c r="O47" s="30" t="inlineStr"/>
       <c r="P47" s="30" t="inlineStr"/>
       <c r="Q47" s="30" t="inlineStr"/>
       <c r="R47" s="30" t="inlineStr"/>
       <c r="S47" s="30" t="inlineStr"/>
-      <c r="T47" s="30" t="inlineStr"/>
-      <c r="U47" s="30" t="inlineStr"/>
-      <c r="V47" s="30" t="inlineStr"/>
+      <c r="T47" s="30" t="inlineStr">
+        <is>
+          <t>14/02/1952</t>
+        </is>
+      </c>
+      <c r="U47" s="30" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="V47" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W47" s="30" t="inlineStr"/>
-      <c r="X47" s="30" t="inlineStr"/>
+      <c r="X47" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y47" s="30" t="inlineStr"/>
       <c r="Z47" s="30" t="inlineStr"/>
-      <c r="AA47" s="30" t="inlineStr"/>
+      <c r="AA47" s="30" t="inlineStr">
+        <is>
+          <t>03/08/2024</t>
+        </is>
+      </c>
       <c r="AB47" s="30" t="inlineStr"/>
       <c r="AC47" s="30" t="inlineStr"/>
       <c r="AD47" s="30" t="inlineStr"/>
@@ -6064,7 +7328,11 @@
       <c r="AR47" s="30" t="inlineStr"/>
       <c r="AS47" s="30" t="inlineStr"/>
       <c r="AT47" s="30" t="inlineStr"/>
-      <c r="AU47" s="30" t="inlineStr"/>
+      <c r="AU47" s="30" t="inlineStr">
+        <is>
+          <t>05/10/2024</t>
+        </is>
+      </c>
       <c r="AV47" s="30" t="inlineStr"/>
       <c r="AW47" s="30" t="inlineStr"/>
       <c r="AX47" s="30" t="inlineStr"/>
@@ -6120,7 +7388,11 @@
           <t>9990000047</t>
         </is>
       </c>
-      <c r="E48" s="30" t="inlineStr"/>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F48" s="30" t="inlineStr"/>
       <c r="G48" s="30" t="inlineStr"/>
       <c r="H48" s="30" t="inlineStr"/>
@@ -6133,20 +7405,36 @@
       </c>
       <c r="L48" s="30" t="inlineStr"/>
       <c r="M48" s="30" t="inlineStr"/>
-      <c r="N48" s="30" t="inlineStr"/>
+      <c r="N48" s="30" t="inlineStr">
+        <is>
+          <t>15/07/2024</t>
+        </is>
+      </c>
       <c r="O48" s="30" t="inlineStr"/>
       <c r="P48" s="30" t="inlineStr"/>
       <c r="Q48" s="30" t="inlineStr"/>
       <c r="R48" s="30" t="inlineStr"/>
       <c r="S48" s="30" t="inlineStr"/>
-      <c r="T48" s="30" t="inlineStr"/>
+      <c r="T48" s="30" t="inlineStr">
+        <is>
+          <t>09/10/1964</t>
+        </is>
+      </c>
       <c r="U48" s="30" t="inlineStr"/>
       <c r="V48" s="30" t="inlineStr"/>
       <c r="W48" s="30" t="inlineStr"/>
-      <c r="X48" s="30" t="inlineStr"/>
+      <c r="X48" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y48" s="30" t="inlineStr"/>
       <c r="Z48" s="30" t="inlineStr"/>
-      <c r="AA48" s="30" t="inlineStr"/>
+      <c r="AA48" s="30" t="inlineStr">
+        <is>
+          <t>22/01/2025</t>
+        </is>
+      </c>
       <c r="AB48" s="30" t="inlineStr"/>
       <c r="AC48" s="30" t="inlineStr"/>
       <c r="AD48" s="30" t="inlineStr"/>
@@ -6222,7 +7510,11 @@
           <t>9990000048</t>
         </is>
       </c>
-      <c r="E49" s="30" t="inlineStr"/>
+      <c r="E49" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F49" s="30" t="inlineStr"/>
       <c r="G49" s="30" t="inlineStr"/>
       <c r="H49" s="30" t="inlineStr"/>
@@ -6235,20 +7527,44 @@
       </c>
       <c r="L49" s="30" t="inlineStr"/>
       <c r="M49" s="30" t="inlineStr"/>
-      <c r="N49" s="30" t="inlineStr"/>
+      <c r="N49" s="30" t="inlineStr">
+        <is>
+          <t>25/03/2025</t>
+        </is>
+      </c>
       <c r="O49" s="30" t="inlineStr"/>
       <c r="P49" s="30" t="inlineStr"/>
       <c r="Q49" s="30" t="inlineStr"/>
       <c r="R49" s="30" t="inlineStr"/>
       <c r="S49" s="30" t="inlineStr"/>
-      <c r="T49" s="30" t="inlineStr"/>
-      <c r="U49" s="30" t="inlineStr"/>
-      <c r="V49" s="30" t="inlineStr"/>
+      <c r="T49" s="30" t="inlineStr">
+        <is>
+          <t>17/11/1959</t>
+        </is>
+      </c>
+      <c r="U49" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V49" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W49" s="30" t="inlineStr"/>
-      <c r="X49" s="30" t="inlineStr"/>
+      <c r="X49" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y49" s="30" t="inlineStr"/>
       <c r="Z49" s="30" t="inlineStr"/>
-      <c r="AA49" s="30" t="inlineStr"/>
+      <c r="AA49" s="30" t="inlineStr">
+        <is>
+          <t>05/05/2024</t>
+        </is>
+      </c>
       <c r="AB49" s="30" t="inlineStr"/>
       <c r="AC49" s="30" t="inlineStr"/>
       <c r="AD49" s="30" t="inlineStr"/>
@@ -6268,7 +7584,11 @@
       <c r="AR49" s="30" t="inlineStr"/>
       <c r="AS49" s="30" t="inlineStr"/>
       <c r="AT49" s="30" t="inlineStr"/>
-      <c r="AU49" s="30" t="inlineStr"/>
+      <c r="AU49" s="30" t="inlineStr">
+        <is>
+          <t>28/12/2024</t>
+        </is>
+      </c>
       <c r="AV49" s="30" t="inlineStr"/>
       <c r="AW49" s="30" t="inlineStr"/>
       <c r="AX49" s="30" t="inlineStr"/>
@@ -6324,7 +7644,11 @@
           <t>9990000049</t>
         </is>
       </c>
-      <c r="E50" s="30" t="inlineStr"/>
+      <c r="E50" s="30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
       <c r="F50" s="30" t="inlineStr"/>
       <c r="G50" s="30" t="inlineStr"/>
       <c r="H50" s="30" t="inlineStr"/>
@@ -6337,20 +7661,44 @@
       </c>
       <c r="L50" s="30" t="inlineStr"/>
       <c r="M50" s="30" t="inlineStr"/>
-      <c r="N50" s="30" t="inlineStr"/>
+      <c r="N50" s="30" t="inlineStr">
+        <is>
+          <t>20/04/2024</t>
+        </is>
+      </c>
       <c r="O50" s="30" t="inlineStr"/>
       <c r="P50" s="30" t="inlineStr"/>
       <c r="Q50" s="30" t="inlineStr"/>
       <c r="R50" s="30" t="inlineStr"/>
       <c r="S50" s="30" t="inlineStr"/>
-      <c r="T50" s="30" t="inlineStr"/>
-      <c r="U50" s="30" t="inlineStr"/>
-      <c r="V50" s="30" t="inlineStr"/>
+      <c r="T50" s="30" t="inlineStr">
+        <is>
+          <t>03/01/1978</t>
+        </is>
+      </c>
+      <c r="U50" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V50" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W50" s="30" t="inlineStr"/>
-      <c r="X50" s="30" t="inlineStr"/>
+      <c r="X50" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y50" s="30" t="inlineStr"/>
       <c r="Z50" s="30" t="inlineStr"/>
-      <c r="AA50" s="30" t="inlineStr"/>
+      <c r="AA50" s="30" t="inlineStr">
+        <is>
+          <t>14/02/2025</t>
+        </is>
+      </c>
       <c r="AB50" s="30" t="inlineStr"/>
       <c r="AC50" s="30" t="inlineStr"/>
       <c r="AD50" s="30" t="inlineStr"/>
@@ -6426,7 +7774,11 @@
           <t>9990000050</t>
         </is>
       </c>
-      <c r="E51" s="30" t="inlineStr"/>
+      <c r="E51" s="30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
       <c r="F51" s="30" t="inlineStr"/>
       <c r="G51" s="30" t="inlineStr"/>
       <c r="H51" s="30" t="inlineStr"/>
@@ -6439,20 +7791,36 @@
       </c>
       <c r="L51" s="30" t="inlineStr"/>
       <c r="M51" s="30" t="inlineStr"/>
-      <c r="N51" s="30" t="inlineStr"/>
+      <c r="N51" s="30" t="inlineStr">
+        <is>
+          <t>17/04/2025</t>
+        </is>
+      </c>
       <c r="O51" s="30" t="inlineStr"/>
       <c r="P51" s="30" t="inlineStr"/>
       <c r="Q51" s="30" t="inlineStr"/>
       <c r="R51" s="30" t="inlineStr"/>
       <c r="S51" s="30" t="inlineStr"/>
-      <c r="T51" s="30" t="inlineStr"/>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>12/05/1945</t>
+        </is>
+      </c>
       <c r="U51" s="30" t="inlineStr"/>
       <c r="V51" s="30" t="inlineStr"/>
       <c r="W51" s="30" t="inlineStr"/>
-      <c r="X51" s="30" t="inlineStr"/>
+      <c r="X51" s="30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="Y51" s="30" t="inlineStr"/>
       <c r="Z51" s="30" t="inlineStr"/>
-      <c r="AA51" s="30" t="inlineStr"/>
+      <c r="AA51" s="30" t="inlineStr">
+        <is>
+          <t>10/01/2025</t>
+        </is>
+      </c>
       <c r="AB51" s="30" t="inlineStr"/>
       <c r="AC51" s="30" t="inlineStr"/>
       <c r="AD51" s="30" t="inlineStr"/>

</xml_diff>